<commit_message>
add missing data quality attributes, add server roles
</commit_message>
<xml_diff>
--- a/examples/shipments-odcs.xlsx
+++ b/examples/shipments-odcs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jakob/entropyData/open-data-contract-standard-excel-template/examples/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E74117F-71BF-6B4A-BCA7-A99069EEEC16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2386967-5C32-014F-86AC-30B7C4876311}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="780" windowWidth="34200" windowHeight="21460" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -57,9 +57,9 @@
     <definedName name="price.priceAmount">Pricing!$B$4</definedName>
     <definedName name="price.priceCurrency">Pricing!$B$5</definedName>
     <definedName name="price.priceUnit">Pricing!$B$6</definedName>
-    <definedName name="quality">Quality!$A$4:$AZ$300</definedName>
+    <definedName name="quality">Quality!$A$4:$BF$300</definedName>
     <definedName name="relationships">Relationships!$A$4:$AZ$300</definedName>
-    <definedName name="roles" localSheetId="7">Roles!$A$4:$AZ$1000</definedName>
+    <definedName name="roles" localSheetId="7">Roles!$C$4:$BB$1000</definedName>
     <definedName name="schema.businessName" localSheetId="2">'Schema shipments'!$B$8</definedName>
     <definedName name="schema.context.instructions" localSheetId="2">'Schema shipments'!$B$13</definedName>
     <definedName name="schema.dataGranularityDescription" localSheetId="2">'Schema shipments'!$B$10</definedName>
@@ -132,7 +132,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="774" uniqueCount="422">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="782" uniqueCount="426">
   <si>
     <t>Fundamentals</t>
   </si>
@@ -836,11 +836,6 @@
   </si>
   <si>
     <t>Roles</t>
-  </si>
-  <si>
-    <t xml:space="preserve">This section lists team members and the history of their relation with this data contract.
-This section lists the roles that a consumer may need to access the dataset depending on the type of access they require.
-</t>
   </si>
   <si>
     <t>Access</t>
@@ -1405,6 +1400,22 @@
   </si>
   <si>
     <t>optional</t>
+  </si>
+  <si>
+    <t>Dimension</t>
+  </si>
+  <si>
+    <t>Method</t>
+  </si>
+  <si>
+    <t>Business Impact</t>
+  </si>
+  <si>
+    <t xml:space="preserve">This section lists the roles that a consumer may need to access the dataset depending on the type of access they require.
+</t>
+  </si>
+  <si>
+    <t>Server Name</t>
   </si>
 </sst>
 </file>
@@ -1611,7 +1622,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1705,6 +1716,7 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -2444,7 +2456,7 @@
   <sheetData>
     <row r="1" spans="1:52" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -2500,7 +2512,7 @@
     </row>
     <row r="2" spans="1:52" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -2610,14 +2622,14 @@
     </row>
     <row r="4" spans="1:52" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="7" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="B4" s="2"/>
       <c r="C4" s="5" t="s">
+        <v>252</v>
+      </c>
+      <c r="D4" s="5" t="s">
         <v>253</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>254</v>
       </c>
       <c r="E4" s="5"/>
       <c r="F4" s="5"/>
@@ -2670,14 +2682,14 @@
     </row>
     <row r="5" spans="1:52" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="7" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="B5" s="2"/>
       <c r="C5" s="5" t="s">
+        <v>252</v>
+      </c>
+      <c r="D5" s="5" t="s">
         <v>253</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>254</v>
       </c>
       <c r="E5" s="5"/>
       <c r="F5" s="5"/>
@@ -2840,14 +2852,14 @@
     </row>
     <row r="8" spans="1:52" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="7" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="B8" s="2"/>
       <c r="C8" s="5" t="s">
+        <v>256</v>
+      </c>
+      <c r="D8" s="5" t="s">
         <v>257</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>258</v>
       </c>
       <c r="E8" s="5"/>
       <c r="F8" s="5"/>
@@ -2954,7 +2966,7 @@
     </row>
     <row r="10" spans="1:52" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="7" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
@@ -3011,7 +3023,7 @@
     <row r="11" spans="1:52" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="2"/>
       <c r="B11" s="2" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="C11" s="5"/>
       <c r="D11" s="5"/>
@@ -3067,7 +3079,7 @@
     <row r="12" spans="1:52" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="2"/>
       <c r="B12" s="2" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="C12" s="5"/>
       <c r="D12" s="5"/>
@@ -3123,7 +3135,7 @@
     <row r="13" spans="1:52" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="2"/>
       <c r="B13" s="2" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="C13" s="5"/>
       <c r="D13" s="5"/>
@@ -3179,7 +3191,7 @@
     <row r="14" spans="1:52" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="2"/>
       <c r="B14" s="2" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="C14" s="5"/>
       <c r="D14" s="5" t="s">
@@ -3237,7 +3249,7 @@
     <row r="15" spans="1:52" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="2"/>
       <c r="B15" s="2" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="C15" s="5" t="s">
         <v>65</v>
@@ -3295,7 +3307,7 @@
     <row r="16" spans="1:52" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="2"/>
       <c r="B16" s="2" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="C16" s="5"/>
       <c r="D16" s="5"/>
@@ -3351,7 +3363,7 @@
     <row r="17" spans="1:52" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="2"/>
       <c r="B17" s="2" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="C17" s="5"/>
       <c r="D17" s="5"/>
@@ -3407,7 +3419,7 @@
     <row r="18" spans="1:52" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="2"/>
       <c r="B18" s="2" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="C18" s="5"/>
       <c r="D18" s="5"/>
@@ -3519,11 +3531,11 @@
     <row r="20" spans="1:52" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="2"/>
       <c r="B20" s="2" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="C20" s="5"/>
       <c r="D20" s="5" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="E20" s="5"/>
       <c r="F20" s="5"/>
@@ -3577,7 +3589,7 @@
     <row r="21" spans="1:52" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="2"/>
       <c r="B21" s="2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="C21" s="5"/>
       <c r="D21" s="5"/>
@@ -3633,7 +3645,7 @@
     <row r="22" spans="1:52" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="2"/>
       <c r="B22" s="2" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="C22" s="5"/>
       <c r="D22" s="5"/>
@@ -3689,7 +3701,7 @@
     <row r="23" spans="1:52" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="2"/>
       <c r="B23" s="2" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="C23" s="5"/>
       <c r="D23" s="5"/>
@@ -3745,11 +3757,11 @@
     <row r="24" spans="1:52" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="2"/>
       <c r="B24" s="2" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="C24" s="5"/>
       <c r="D24" s="5" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="E24" s="5"/>
       <c r="F24" s="5"/>
@@ -3803,10 +3815,10 @@
     <row r="25" spans="1:52" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="2"/>
       <c r="B25" s="2" t="s">
+        <v>274</v>
+      </c>
+      <c r="C25" s="5" t="s">
         <v>275</v>
-      </c>
-      <c r="C25" s="5" t="s">
-        <v>276</v>
       </c>
       <c r="D25" s="5"/>
       <c r="E25" s="5"/>
@@ -3861,7 +3873,7 @@
     <row r="26" spans="1:52" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="2"/>
       <c r="B26" s="2" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="C26" s="5"/>
       <c r="D26" s="5"/>
@@ -3917,7 +3929,7 @@
     <row r="27" spans="1:52" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="2"/>
       <c r="B27" s="2" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="C27" s="5"/>
       <c r="D27" s="5"/>
@@ -3977,7 +3989,7 @@
       </c>
       <c r="C28" s="5"/>
       <c r="D28" s="5" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="E28" s="5"/>
       <c r="F28" s="5"/>
@@ -4031,7 +4043,7 @@
     <row r="29" spans="1:52" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="2"/>
       <c r="B29" s="2" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="C29" s="5"/>
       <c r="D29" s="5"/>
@@ -4087,7 +4099,7 @@
     <row r="30" spans="1:52" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="2"/>
       <c r="B30" s="2" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="C30" s="5"/>
       <c r="D30" s="5"/>
@@ -4143,7 +4155,7 @@
     <row r="31" spans="1:52" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="2"/>
       <c r="B31" s="2" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="C31" s="5"/>
       <c r="D31" s="5"/>
@@ -4199,7 +4211,7 @@
     <row r="32" spans="1:52" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="2"/>
       <c r="B32" s="2" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="C32" s="5"/>
       <c r="D32" s="5"/>
@@ -4255,7 +4267,7 @@
     <row r="33" spans="1:52" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="2"/>
       <c r="B33" s="2" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="C33" s="5"/>
       <c r="D33" s="5"/>
@@ -4368,10 +4380,10 @@
         <v>6</v>
       </c>
       <c r="C35" s="5" t="s">
+        <v>252</v>
+      </c>
+      <c r="D35" s="5" t="s">
         <v>253</v>
-      </c>
-      <c r="D35" s="5" t="s">
-        <v>254</v>
       </c>
       <c r="E35" s="5"/>
       <c r="F35" s="5"/>
@@ -4478,7 +4490,7 @@
     </row>
     <row r="37" spans="1:52" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="7" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="B37" s="2"/>
       <c r="C37" s="2"/>
@@ -13416,18 +13428,18 @@
   <sheetData>
     <row r="1" spans="1:2" s="2" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="2" spans="1:2" s="2" customFormat="1" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="3" spans="1:2" s="2" customFormat="1" ht="16" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="4" spans="1:2" s="2" customFormat="1" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="7" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="B4" s="5">
         <v>1</v>
@@ -13435,23 +13447,23 @@
     </row>
     <row r="5" spans="1:2" s="2" customFormat="1" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="7" t="s">
+        <v>288</v>
+      </c>
+      <c r="B5" s="5" t="s">
         <v>289</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>290</v>
       </c>
     </row>
     <row r="6" spans="1:2" s="2" customFormat="1" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="7" t="s">
+        <v>290</v>
+      </c>
+      <c r="B6" s="5" t="s">
         <v>291</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>292</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="7" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="B7" s="5"/>
     </row>
@@ -13482,13 +13494,13 @@
   <sheetData>
     <row r="1" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="29" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="B1" s="29"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="31" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="B2" s="31"/>
     </row>
@@ -13501,10 +13513,10 @@
         <v>213</v>
       </c>
       <c r="B4" s="32" t="s">
+        <v>295</v>
+      </c>
+      <c r="C4" s="33" t="s">
         <v>296</v>
-      </c>
-      <c r="C4" s="33" t="s">
-        <v>297</v>
       </c>
       <c r="D4" s="33" t="s">
         <v>60</v>
@@ -13518,14 +13530,14 @@
     </row>
     <row r="5" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A5" s="17" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="B5" s="17"/>
       <c r="C5" s="15" t="s">
+        <v>298</v>
+      </c>
+      <c r="D5" s="15" t="s">
         <v>299</v>
-      </c>
-      <c r="D5" s="15" t="s">
-        <v>300</v>
       </c>
       <c r="E5" s="15"/>
       <c r="F5" s="17"/>
@@ -13536,42 +13548,42 @@
       </c>
       <c r="B6" s="17"/>
       <c r="C6" s="15" t="s">
+        <v>300</v>
+      </c>
+      <c r="D6" s="15" t="s">
         <v>301</v>
-      </c>
-      <c r="D6" s="15" t="s">
-        <v>302</v>
       </c>
       <c r="E6" s="15"/>
       <c r="F6" s="17"/>
     </row>
     <row r="7" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A7" s="17" t="s">
+        <v>302</v>
+      </c>
+      <c r="B7" s="17" t="s">
         <v>303</v>
       </c>
-      <c r="B7" s="17" t="s">
-        <v>304</v>
-      </c>
       <c r="C7" s="15" t="s">
+        <v>300</v>
+      </c>
+      <c r="D7" s="15" t="s">
         <v>301</v>
-      </c>
-      <c r="D7" s="15" t="s">
-        <v>302</v>
       </c>
       <c r="E7" s="15"/>
       <c r="F7" s="17"/>
     </row>
     <row r="8" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A8" s="17" t="s">
+        <v>304</v>
+      </c>
+      <c r="B8" s="17" t="s">
+        <v>245</v>
+      </c>
+      <c r="C8" s="15" t="s">
         <v>305</v>
       </c>
-      <c r="B8" s="17" t="s">
-        <v>246</v>
-      </c>
-      <c r="C8" s="15" t="s">
-        <v>306</v>
-      </c>
       <c r="D8" s="15" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="E8" s="15"/>
       <c r="F8" s="17"/>
@@ -13713,13 +13725,13 @@
   <sheetData>
     <row r="1" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="29" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="B1" s="29"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" s="31" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="B2" s="31"/>
     </row>
@@ -13737,13 +13749,13 @@
         <v>213</v>
       </c>
       <c r="B4" s="32" t="s">
+        <v>308</v>
+      </c>
+      <c r="C4" s="33" t="s">
         <v>309</v>
       </c>
-      <c r="C4" s="33" t="s">
+      <c r="D4" s="33" t="s">
         <v>310</v>
-      </c>
-      <c r="D4" s="33" t="s">
-        <v>311</v>
       </c>
       <c r="E4" s="33" t="s">
         <v>28</v>
@@ -13757,20 +13769,20 @@
     </row>
     <row r="5" spans="1:9" ht="34" x14ac:dyDescent="0.2">
       <c r="A5" s="17" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="B5" s="17"/>
       <c r="C5" s="15" t="s">
+        <v>312</v>
+      </c>
+      <c r="D5" s="15" t="s">
         <v>313</v>
       </c>
-      <c r="D5" s="15" t="s">
+      <c r="E5" s="15" t="s">
         <v>314</v>
       </c>
-      <c r="E5" s="15" t="s">
+      <c r="F5" s="17" t="s">
         <v>315</v>
-      </c>
-      <c r="F5" s="17" t="s">
-        <v>316</v>
       </c>
       <c r="G5" s="15"/>
       <c r="H5" s="15"/>
@@ -13778,16 +13790,16 @@
     </row>
     <row r="6" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="A6" s="17" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="B6" s="17"/>
       <c r="C6" s="15" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="D6" s="15"/>
       <c r="E6" s="15"/>
       <c r="F6" s="17" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="G6" s="15"/>
       <c r="H6" s="15"/>
@@ -13991,13 +14003,13 @@
   <sheetData>
     <row r="1" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="29" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="B1" s="29"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" s="31" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="B2" s="31"/>
     </row>
@@ -14015,10 +14027,10 @@
         <v>213</v>
       </c>
       <c r="B4" s="32" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="C4" s="33" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="D4" s="33" t="s">
         <v>28</v>
@@ -14032,15 +14044,15 @@
     </row>
     <row r="5" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A5" s="17" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="B5" s="17"/>
       <c r="C5" s="15" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="D5" s="15"/>
       <c r="E5" s="17" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="F5" s="15"/>
       <c r="G5" s="15"/>
@@ -14048,13 +14060,13 @@
     </row>
     <row r="6" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A6" s="17" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="B6" s="17" t="s">
         <v>59</v>
       </c>
       <c r="C6" s="15" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="D6" s="15"/>
       <c r="E6" s="17"/>
@@ -14247,13 +14259,13 @@
   <sheetData>
     <row r="1" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="29" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="B1" s="29"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" s="31" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="B2" s="31"/>
     </row>
@@ -14274,10 +14286,10 @@
         <v>74</v>
       </c>
       <c r="C4" s="33" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="D4" s="33" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="E4" s="33" t="s">
         <v>21</v>
@@ -14300,16 +14312,16 @@
         <v>142</v>
       </c>
       <c r="C5" s="15" t="s">
+        <v>326</v>
+      </c>
+      <c r="D5" s="15" t="s">
+        <v>326</v>
+      </c>
+      <c r="E5" s="15" t="s">
         <v>327</v>
       </c>
-      <c r="D5" s="15" t="s">
-        <v>327</v>
-      </c>
-      <c r="E5" s="15" t="s">
+      <c r="F5" s="17" t="s">
         <v>328</v>
-      </c>
-      <c r="F5" s="17" t="s">
-        <v>329</v>
       </c>
       <c r="G5" s="17"/>
       <c r="H5" s="15"/>
@@ -14324,13 +14336,13 @@
         <v>142</v>
       </c>
       <c r="C6" s="15" t="s">
+        <v>329</v>
+      </c>
+      <c r="D6" s="15" t="s">
+        <v>329</v>
+      </c>
+      <c r="E6" s="15" t="s">
         <v>330</v>
-      </c>
-      <c r="D6" s="15" t="s">
-        <v>330</v>
-      </c>
-      <c r="E6" s="15" t="s">
-        <v>331</v>
       </c>
       <c r="F6" s="17"/>
       <c r="G6" s="17"/>
@@ -14346,13 +14358,13 @@
         <v>142</v>
       </c>
       <c r="C7" s="15" t="s">
+        <v>331</v>
+      </c>
+      <c r="D7" s="15" t="s">
+        <v>331</v>
+      </c>
+      <c r="E7" s="15" t="s">
         <v>332</v>
-      </c>
-      <c r="D7" s="15" t="s">
-        <v>332</v>
-      </c>
-      <c r="E7" s="15" t="s">
-        <v>333</v>
       </c>
       <c r="F7" s="17"/>
       <c r="G7" s="17"/>
@@ -14371,7 +14383,7 @@
         <v>177</v>
       </c>
       <c r="D8" s="15" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="E8" s="15"/>
       <c r="F8" s="17"/>
@@ -14388,10 +14400,10 @@
         <v>175</v>
       </c>
       <c r="C9" s="15" t="s">
+        <v>334</v>
+      </c>
+      <c r="D9" s="15" t="s">
         <v>335</v>
-      </c>
-      <c r="D9" s="15" t="s">
-        <v>336</v>
       </c>
       <c r="E9" s="15"/>
       <c r="F9" s="17"/>
@@ -14408,10 +14420,10 @@
         <v>175</v>
       </c>
       <c r="C10" s="15" t="s">
+        <v>336</v>
+      </c>
+      <c r="D10" s="15" t="s">
         <v>337</v>
-      </c>
-      <c r="D10" s="15" t="s">
-        <v>338</v>
       </c>
       <c r="E10" s="15"/>
       <c r="F10" s="17"/>
@@ -14585,13 +14597,13 @@
   <sheetData>
     <row r="1" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="29" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="B1" s="29"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2" s="31" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="B2" s="31"/>
     </row>
@@ -14612,13 +14624,13 @@
         <v>74</v>
       </c>
       <c r="C4" s="33" t="s">
+        <v>340</v>
+      </c>
+      <c r="D4" s="33" t="s">
         <v>341</v>
       </c>
-      <c r="D4" s="33" t="s">
+      <c r="E4" s="33" t="s">
         <v>342</v>
-      </c>
-      <c r="E4" s="33" t="s">
-        <v>343</v>
       </c>
       <c r="F4" s="32" t="s">
         <v>12</v>
@@ -14639,17 +14651,17 @@
       </c>
       <c r="B5" s="17"/>
       <c r="C5" s="15" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="D5" s="15"/>
       <c r="E5" s="15" t="s">
+        <v>344</v>
+      </c>
+      <c r="F5" s="17" t="s">
         <v>345</v>
       </c>
-      <c r="F5" s="17" t="s">
+      <c r="G5" s="17" t="s">
         <v>346</v>
-      </c>
-      <c r="G5" s="17" t="s">
-        <v>347</v>
       </c>
       <c r="H5" s="17"/>
       <c r="I5" s="15"/>
@@ -14662,10 +14674,10 @@
       </c>
       <c r="B6" s="17"/>
       <c r="C6" s="15" t="s">
+        <v>347</v>
+      </c>
+      <c r="D6" s="15" t="s">
         <v>348</v>
-      </c>
-      <c r="D6" s="15" t="s">
-        <v>349</v>
       </c>
       <c r="E6" s="15"/>
       <c r="F6" s="17"/>
@@ -14683,11 +14695,11 @@
         <v>109</v>
       </c>
       <c r="C7" s="15" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="D7" s="15"/>
       <c r="E7" s="15" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="F7" s="17"/>
       <c r="G7" s="17"/>
@@ -14704,7 +14716,7 @@
         <v>132</v>
       </c>
       <c r="C8" s="15" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="D8" s="15"/>
       <c r="E8" s="15"/>
@@ -14920,12 +14932,12 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" s="4" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
@@ -14933,19 +14945,19 @@
         <v>213</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="C4" s="9" t="s">
         <v>74</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="E4" s="10" t="s">
         <v>21</v>
       </c>
       <c r="F4" s="10" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="G4" s="10" t="s">
         <v>6</v>
@@ -14953,11 +14965,11 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" s="5" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="B5" s="5"/>
       <c r="C5" s="5" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="D5" s="5" t="str">
         <f>IF(owner &lt;&gt; "", owner, "")</f>
@@ -14969,14 +14981,14 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" s="5" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="B6" s="5"/>
       <c r="C6" s="5" t="s">
+        <v>357</v>
+      </c>
+      <c r="D6" s="5" t="s">
         <v>358</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>359</v>
       </c>
       <c r="E6" s="5"/>
       <c r="F6" s="5"/>
@@ -14984,18 +14996,18 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" s="5" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="B7" s="5"/>
       <c r="C7" s="5" t="s">
+        <v>359</v>
+      </c>
+      <c r="D7" s="5" t="s">
         <v>360</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>361</v>
       </c>
       <c r="E7" s="5"/>
       <c r="F7" s="5" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="G7" s="5"/>
     </row>
@@ -15005,10 +15017,10 @@
       </c>
       <c r="B8" s="5"/>
       <c r="C8" s="5" t="s">
+        <v>362</v>
+      </c>
+      <c r="D8" s="5" t="s">
         <v>363</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>364</v>
       </c>
       <c r="E8" s="5"/>
       <c r="F8" s="5"/>
@@ -15019,13 +15031,13 @@
         <v>74</v>
       </c>
       <c r="B9" s="5" t="s">
+        <v>364</v>
+      </c>
+      <c r="C9" s="5" t="s">
         <v>365</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="D9" s="5" t="s">
         <v>366</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>367</v>
       </c>
       <c r="E9" s="5"/>
       <c r="F9" s="5"/>
@@ -15036,32 +15048,32 @@
         <v>74</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="C10" s="5" t="s">
+        <v>367</v>
+      </c>
+      <c r="D10" s="5" t="s">
         <v>368</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>369</v>
       </c>
       <c r="E10" s="5"/>
       <c r="F10" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="G10" s="5"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" s="5" t="s">
+        <v>370</v>
+      </c>
+      <c r="B11" s="5" t="s">
         <v>371</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="C11" s="5" t="s">
         <v>372</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="D11" s="5" t="s">
         <v>373</v>
-      </c>
-      <c r="D11" s="5" t="s">
-        <v>374</v>
       </c>
       <c r="E11" s="5"/>
       <c r="F11" s="5"/>
@@ -15069,20 +15081,20 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" s="5" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="C12" s="5" t="s">
+        <v>374</v>
+      </c>
+      <c r="D12" s="5" t="s">
         <v>375</v>
-      </c>
-      <c r="D12" s="5" t="s">
-        <v>376</v>
       </c>
       <c r="E12" s="5"/>
       <c r="F12" s="5" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="G12" s="5"/>
     </row>
@@ -15185,341 +15197,341 @@
   <sheetData>
     <row r="1" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
+        <v>377</v>
+      </c>
+      <c r="B1" t="s">
         <v>378</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>379</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>380</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
+        <v>256</v>
+      </c>
+      <c r="F1" t="s">
         <v>381</v>
       </c>
-      <c r="E1" t="s">
+      <c r="G1" t="s">
+        <v>382</v>
+      </c>
+      <c r="H1" t="s">
+        <v>383</v>
+      </c>
+      <c r="I1" t="s">
+        <v>384</v>
+      </c>
+      <c r="J1" t="s">
+        <v>385</v>
+      </c>
+      <c r="K1" t="s">
+        <v>386</v>
+      </c>
+      <c r="L1" t="s">
+        <v>387</v>
+      </c>
+      <c r="M1" t="s">
+        <v>388</v>
+      </c>
+      <c r="N1" t="s">
+        <v>389</v>
+      </c>
+      <c r="O1" t="s">
+        <v>390</v>
+      </c>
+      <c r="P1" t="s">
+        <v>391</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>392</v>
+      </c>
+      <c r="R1" t="s">
+        <v>393</v>
+      </c>
+      <c r="S1" t="s">
+        <v>394</v>
+      </c>
+      <c r="T1" t="s">
+        <v>395</v>
+      </c>
+      <c r="U1" t="s">
+        <v>396</v>
+      </c>
+      <c r="V1" t="s">
+        <v>397</v>
+      </c>
+      <c r="W1" t="s">
+        <v>398</v>
+      </c>
+      <c r="X1" t="s">
+        <v>399</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>400</v>
+      </c>
+      <c r="Z1" t="s">
+        <v>401</v>
+      </c>
+      <c r="AA1" t="s">
+        <v>402</v>
+      </c>
+      <c r="AB1" t="s">
+        <v>403</v>
+      </c>
+      <c r="AC1" t="s">
         <v>257</v>
       </c>
-      <c r="F1" t="s">
-        <v>382</v>
-      </c>
-      <c r="G1" t="s">
-        <v>383</v>
-      </c>
-      <c r="H1" t="s">
-        <v>384</v>
-      </c>
-      <c r="I1" t="s">
-        <v>385</v>
-      </c>
-      <c r="J1" t="s">
-        <v>386</v>
-      </c>
-      <c r="K1" t="s">
-        <v>387</v>
-      </c>
-      <c r="L1" t="s">
-        <v>388</v>
-      </c>
-      <c r="M1" t="s">
-        <v>389</v>
-      </c>
-      <c r="N1" t="s">
-        <v>390</v>
-      </c>
-      <c r="O1" t="s">
-        <v>391</v>
-      </c>
-      <c r="P1" t="s">
-        <v>392</v>
-      </c>
-      <c r="Q1" t="s">
-        <v>393</v>
-      </c>
-      <c r="R1" t="s">
-        <v>394</v>
-      </c>
-      <c r="S1" t="s">
-        <v>395</v>
-      </c>
-      <c r="T1" t="s">
-        <v>396</v>
-      </c>
-      <c r="U1" t="s">
-        <v>397</v>
-      </c>
-      <c r="V1" t="s">
-        <v>398</v>
-      </c>
-      <c r="W1" t="s">
-        <v>399</v>
-      </c>
-      <c r="X1" t="s">
-        <v>400</v>
-      </c>
-      <c r="Y1" t="s">
-        <v>401</v>
-      </c>
-      <c r="Z1" t="s">
-        <v>402</v>
-      </c>
-      <c r="AA1" t="s">
-        <v>403</v>
-      </c>
-      <c r="AB1" t="s">
+      <c r="AD1" t="s">
         <v>404</v>
       </c>
-      <c r="AC1" t="s">
-        <v>258</v>
-      </c>
-      <c r="AD1" t="s">
+      <c r="AE1" t="s">
         <v>405</v>
       </c>
-      <c r="AE1" t="s">
+      <c r="AF1" t="s">
         <v>406</v>
       </c>
-      <c r="AF1" t="s">
+      <c r="AG1" t="s">
         <v>407</v>
       </c>
-      <c r="AG1" t="s">
+      <c r="AH1" t="s">
         <v>408</v>
       </c>
-      <c r="AH1" t="s">
+      <c r="AI1" t="s">
         <v>409</v>
       </c>
-      <c r="AI1" t="s">
+      <c r="AJ1" t="s">
+        <v>369</v>
+      </c>
+      <c r="AK1" t="s">
         <v>410</v>
       </c>
-      <c r="AJ1" t="s">
-        <v>370</v>
-      </c>
-      <c r="AK1" t="s">
+      <c r="AL1" t="s">
         <v>411</v>
       </c>
-      <c r="AL1" t="s">
+      <c r="AM1" t="s">
         <v>412</v>
       </c>
-      <c r="AM1" t="s">
+      <c r="AN1" t="s">
         <v>413</v>
       </c>
-      <c r="AN1" t="s">
+      <c r="AO1" t="s">
         <v>414</v>
       </c>
-      <c r="AO1" t="s">
+      <c r="AP1" t="s">
         <v>415</v>
       </c>
-      <c r="AP1" t="s">
+      <c r="AQ1" t="s">
         <v>416</v>
       </c>
-      <c r="AQ1" t="s">
+      <c r="AR1" t="s">
         <v>417</v>
       </c>
-      <c r="AR1" t="s">
+      <c r="AS1" t="s">
         <v>418</v>
-      </c>
-      <c r="AS1" t="s">
-        <v>419</v>
       </c>
     </row>
     <row r="2" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="N2" t="s">
+        <v>419</v>
+      </c>
+      <c r="AG2" t="s">
         <v>420</v>
       </c>
-      <c r="AG2" t="s">
-        <v>421</v>
-      </c>
       <c r="AJ2" t="s">
+        <v>419</v>
+      </c>
+      <c r="AS2" t="s">
         <v>420</v>
-      </c>
-      <c r="AS2" t="s">
-        <v>421</v>
       </c>
     </row>
     <row r="3" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="C3" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="H3" t="s">
+        <v>419</v>
+      </c>
+      <c r="S3" t="s">
+        <v>419</v>
+      </c>
+      <c r="AE3" t="s">
         <v>420</v>
       </c>
-      <c r="S3" t="s">
+      <c r="AN3" t="s">
+        <v>419</v>
+      </c>
+      <c r="AS3" t="s">
         <v>420</v>
-      </c>
-      <c r="AE3" t="s">
-        <v>421</v>
-      </c>
-      <c r="AN3" t="s">
-        <v>420</v>
-      </c>
-      <c r="AS3" t="s">
-        <v>421</v>
       </c>
     </row>
     <row r="4" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="S4" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
     </row>
     <row r="5" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="F5" t="s">
+        <v>419</v>
+      </c>
+      <c r="G5" t="s">
+        <v>419</v>
+      </c>
+      <c r="I5" t="s">
         <v>420</v>
       </c>
-      <c r="G5" t="s">
+      <c r="K5" t="s">
+        <v>419</v>
+      </c>
+      <c r="M5" t="s">
+        <v>419</v>
+      </c>
+      <c r="N5" t="s">
+        <v>419</v>
+      </c>
+      <c r="O5" t="s">
         <v>420</v>
       </c>
-      <c r="I5" t="s">
-        <v>421</v>
-      </c>
-      <c r="K5" t="s">
+      <c r="P5" t="s">
+        <v>419</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>419</v>
+      </c>
+      <c r="R5" t="s">
+        <v>419</v>
+      </c>
+      <c r="T5" t="s">
+        <v>419</v>
+      </c>
+      <c r="U5" t="s">
+        <v>419</v>
+      </c>
+      <c r="V5" t="s">
+        <v>419</v>
+      </c>
+      <c r="Z5" t="s">
+        <v>419</v>
+      </c>
+      <c r="AB5" t="s">
+        <v>419</v>
+      </c>
+      <c r="AC5" t="s">
+        <v>419</v>
+      </c>
+      <c r="AD5" t="s">
+        <v>419</v>
+      </c>
+      <c r="AG5" t="s">
+        <v>419</v>
+      </c>
+      <c r="AJ5" t="s">
+        <v>419</v>
+      </c>
+      <c r="AK5" t="s">
+        <v>419</v>
+      </c>
+      <c r="AL5" t="s">
+        <v>419</v>
+      </c>
+      <c r="AM5" t="s">
         <v>420</v>
       </c>
-      <c r="M5" t="s">
+      <c r="AO5" t="s">
+        <v>419</v>
+      </c>
+      <c r="AP5" t="s">
+        <v>419</v>
+      </c>
+      <c r="AQ5" t="s">
+        <v>419</v>
+      </c>
+      <c r="AR5" t="s">
+        <v>419</v>
+      </c>
+      <c r="AS5" t="s">
         <v>420</v>
-      </c>
-      <c r="N5" t="s">
-        <v>420</v>
-      </c>
-      <c r="O5" t="s">
-        <v>421</v>
-      </c>
-      <c r="P5" t="s">
-        <v>420</v>
-      </c>
-      <c r="Q5" t="s">
-        <v>420</v>
-      </c>
-      <c r="R5" t="s">
-        <v>420</v>
-      </c>
-      <c r="T5" t="s">
-        <v>420</v>
-      </c>
-      <c r="U5" t="s">
-        <v>420</v>
-      </c>
-      <c r="V5" t="s">
-        <v>420</v>
-      </c>
-      <c r="Z5" t="s">
-        <v>420</v>
-      </c>
-      <c r="AB5" t="s">
-        <v>420</v>
-      </c>
-      <c r="AC5" t="s">
-        <v>420</v>
-      </c>
-      <c r="AD5" t="s">
-        <v>420</v>
-      </c>
-      <c r="AG5" t="s">
-        <v>420</v>
-      </c>
-      <c r="AJ5" t="s">
-        <v>420</v>
-      </c>
-      <c r="AK5" t="s">
-        <v>420</v>
-      </c>
-      <c r="AL5" t="s">
-        <v>420</v>
-      </c>
-      <c r="AM5" t="s">
-        <v>421</v>
-      </c>
-      <c r="AO5" t="s">
-        <v>420</v>
-      </c>
-      <c r="AP5" t="s">
-        <v>420</v>
-      </c>
-      <c r="AQ5" t="s">
-        <v>420</v>
-      </c>
-      <c r="AR5" t="s">
-        <v>420</v>
-      </c>
-      <c r="AS5" t="s">
-        <v>421</v>
       </c>
     </row>
     <row r="6" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="E6" t="s">
+        <v>419</v>
+      </c>
+      <c r="AS6" t="s">
         <v>420</v>
-      </c>
-      <c r="AS6" t="s">
-        <v>421</v>
       </c>
     </row>
     <row r="7" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="D7" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="AH7" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="AI7" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="AS7" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
     </row>
     <row r="8" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="D8" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="N8" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="W8" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="X8" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="Y8" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="AH8" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="AI8" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="AS8" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
     </row>
     <row r="9" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="AH9" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="AS9" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
     </row>
     <row r="10" spans="1:45" x14ac:dyDescent="0.2">
@@ -15527,299 +15539,299 @@
         <v>96</v>
       </c>
       <c r="D10" t="s">
+        <v>419</v>
+      </c>
+      <c r="N10" t="s">
         <v>420</v>
       </c>
-      <c r="N10" t="s">
-        <v>421</v>
-      </c>
       <c r="W10" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="X10" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="Y10" t="s">
+        <v>419</v>
+      </c>
+      <c r="AH10" t="s">
         <v>420</v>
       </c>
-      <c r="AH10" t="s">
-        <v>421</v>
-      </c>
       <c r="AI10" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="AS10" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
     </row>
     <row r="11" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="F11" t="s">
+        <v>419</v>
+      </c>
+      <c r="G11" t="s">
+        <v>419</v>
+      </c>
+      <c r="H11" t="s">
         <v>420</v>
       </c>
-      <c r="G11" t="s">
+      <c r="I11" t="s">
+        <v>419</v>
+      </c>
+      <c r="J11" t="s">
+        <v>419</v>
+      </c>
+      <c r="L11" t="s">
+        <v>419</v>
+      </c>
+      <c r="M11" t="s">
         <v>420</v>
       </c>
-      <c r="H11" t="s">
-        <v>421</v>
-      </c>
-      <c r="I11" t="s">
+      <c r="O11" t="s">
+        <v>419</v>
+      </c>
+      <c r="P11" t="s">
+        <v>419</v>
+      </c>
+      <c r="Q11" t="s">
+        <v>419</v>
+      </c>
+      <c r="R11" t="s">
+        <v>419</v>
+      </c>
+      <c r="T11" t="s">
+        <v>419</v>
+      </c>
+      <c r="U11" t="s">
+        <v>419</v>
+      </c>
+      <c r="V11" t="s">
+        <v>419</v>
+      </c>
+      <c r="W11" t="s">
+        <v>419</v>
+      </c>
+      <c r="Z11" t="s">
+        <v>419</v>
+      </c>
+      <c r="AA11" t="s">
+        <v>419</v>
+      </c>
+      <c r="AB11" t="s">
         <v>420</v>
       </c>
-      <c r="J11" t="s">
+      <c r="AC11" t="s">
+        <v>419</v>
+      </c>
+      <c r="AD11" t="s">
+        <v>419</v>
+      </c>
+      <c r="AE11" t="s">
+        <v>419</v>
+      </c>
+      <c r="AG11" t="s">
         <v>420</v>
       </c>
-      <c r="L11" t="s">
+      <c r="AJ11" t="s">
+        <v>419</v>
+      </c>
+      <c r="AK11" t="s">
+        <v>419</v>
+      </c>
+      <c r="AL11" t="s">
+        <v>419</v>
+      </c>
+      <c r="AM11" t="s">
+        <v>419</v>
+      </c>
+      <c r="AN11" t="s">
+        <v>419</v>
+      </c>
+      <c r="AO11" t="s">
+        <v>419</v>
+      </c>
+      <c r="AP11" t="s">
         <v>420</v>
       </c>
-      <c r="M11" t="s">
-        <v>421</v>
-      </c>
-      <c r="O11" t="s">
+      <c r="AQ11" t="s">
+        <v>419</v>
+      </c>
+      <c r="AR11" t="s">
+        <v>419</v>
+      </c>
+      <c r="AS11" t="s">
         <v>420</v>
-      </c>
-      <c r="P11" t="s">
-        <v>420</v>
-      </c>
-      <c r="Q11" t="s">
-        <v>420</v>
-      </c>
-      <c r="R11" t="s">
-        <v>420</v>
-      </c>
-      <c r="T11" t="s">
-        <v>420</v>
-      </c>
-      <c r="U11" t="s">
-        <v>420</v>
-      </c>
-      <c r="V11" t="s">
-        <v>420</v>
-      </c>
-      <c r="W11" t="s">
-        <v>420</v>
-      </c>
-      <c r="Z11" t="s">
-        <v>420</v>
-      </c>
-      <c r="AA11" t="s">
-        <v>420</v>
-      </c>
-      <c r="AB11" t="s">
-        <v>421</v>
-      </c>
-      <c r="AC11" t="s">
-        <v>420</v>
-      </c>
-      <c r="AD11" t="s">
-        <v>420</v>
-      </c>
-      <c r="AE11" t="s">
-        <v>420</v>
-      </c>
-      <c r="AG11" t="s">
-        <v>421</v>
-      </c>
-      <c r="AJ11" t="s">
-        <v>420</v>
-      </c>
-      <c r="AK11" t="s">
-        <v>420</v>
-      </c>
-      <c r="AL11" t="s">
-        <v>420</v>
-      </c>
-      <c r="AM11" t="s">
-        <v>420</v>
-      </c>
-      <c r="AN11" t="s">
-        <v>420</v>
-      </c>
-      <c r="AO11" t="s">
-        <v>420</v>
-      </c>
-      <c r="AP11" t="s">
-        <v>421</v>
-      </c>
-      <c r="AQ11" t="s">
-        <v>420</v>
-      </c>
-      <c r="AR11" t="s">
-        <v>420</v>
-      </c>
-      <c r="AS11" t="s">
-        <v>421</v>
       </c>
     </row>
     <row r="12" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="B12" t="s">
+        <v>419</v>
+      </c>
+      <c r="D12" t="s">
+        <v>419</v>
+      </c>
+      <c r="N12" t="s">
         <v>420</v>
       </c>
-      <c r="D12" t="s">
+      <c r="AH12" t="s">
+        <v>419</v>
+      </c>
+      <c r="AI12" t="s">
+        <v>419</v>
+      </c>
+      <c r="AS12" t="s">
         <v>420</v>
-      </c>
-      <c r="N12" t="s">
-        <v>421</v>
-      </c>
-      <c r="AH12" t="s">
-        <v>420</v>
-      </c>
-      <c r="AI12" t="s">
-        <v>420</v>
-      </c>
-      <c r="AS12" t="s">
-        <v>421</v>
       </c>
     </row>
     <row r="13" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="S13" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
     </row>
     <row r="14" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="Y14" t="s">
+        <v>419</v>
+      </c>
+      <c r="AS14" t="s">
         <v>420</v>
-      </c>
-      <c r="AS14" t="s">
-        <v>421</v>
       </c>
     </row>
     <row r="15" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F15" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="G15" t="s">
+        <v>419</v>
+      </c>
+      <c r="I15" t="s">
+        <v>419</v>
+      </c>
+      <c r="J15" t="s">
+        <v>419</v>
+      </c>
+      <c r="L15" t="s">
         <v>420</v>
       </c>
-      <c r="I15" t="s">
+      <c r="M15" t="s">
         <v>420</v>
       </c>
-      <c r="J15" t="s">
+      <c r="O15" t="s">
         <v>420</v>
       </c>
-      <c r="L15" t="s">
-        <v>421</v>
-      </c>
-      <c r="M15" t="s">
-        <v>421</v>
-      </c>
-      <c r="O15" t="s">
-        <v>421</v>
-      </c>
       <c r="P15" t="s">
+        <v>419</v>
+      </c>
+      <c r="Q15" t="s">
+        <v>419</v>
+      </c>
+      <c r="R15" t="s">
         <v>420</v>
       </c>
-      <c r="Q15" t="s">
+      <c r="T15" t="s">
         <v>420</v>
       </c>
-      <c r="R15" t="s">
-        <v>421</v>
-      </c>
-      <c r="T15" t="s">
-        <v>421</v>
-      </c>
       <c r="U15" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="V15" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="Z15" t="s">
+        <v>419</v>
+      </c>
+      <c r="AA15" t="s">
+        <v>419</v>
+      </c>
+      <c r="AB15" t="s">
         <v>420</v>
       </c>
-      <c r="AA15" t="s">
+      <c r="AC15" t="s">
+        <v>419</v>
+      </c>
+      <c r="AD15" t="s">
+        <v>419</v>
+      </c>
+      <c r="AJ15" t="s">
+        <v>419</v>
+      </c>
+      <c r="AK15" t="s">
         <v>420</v>
       </c>
-      <c r="AB15" t="s">
-        <v>421</v>
-      </c>
-      <c r="AC15" t="s">
+      <c r="AL15" t="s">
+        <v>419</v>
+      </c>
+      <c r="AM15" t="s">
         <v>420</v>
       </c>
-      <c r="AD15" t="s">
+      <c r="AN15" t="s">
+        <v>419</v>
+      </c>
+      <c r="AO15" t="s">
         <v>420</v>
       </c>
-      <c r="AJ15" t="s">
+      <c r="AP15" t="s">
         <v>420</v>
       </c>
-      <c r="AK15" t="s">
-        <v>421</v>
-      </c>
-      <c r="AL15" t="s">
+      <c r="AQ15" t="s">
+        <v>419</v>
+      </c>
+      <c r="AR15" t="s">
         <v>420</v>
       </c>
-      <c r="AM15" t="s">
-        <v>421</v>
-      </c>
-      <c r="AN15" t="s">
+      <c r="AS15" t="s">
         <v>420</v>
-      </c>
-      <c r="AO15" t="s">
-        <v>421</v>
-      </c>
-      <c r="AP15" t="s">
-        <v>421</v>
-      </c>
-      <c r="AQ15" t="s">
-        <v>420</v>
-      </c>
-      <c r="AR15" t="s">
-        <v>421</v>
-      </c>
-      <c r="AS15" t="s">
-        <v>421</v>
       </c>
     </row>
     <row r="16" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="E16" t="s">
+        <v>419</v>
+      </c>
+      <c r="AF16" t="s">
+        <v>419</v>
+      </c>
+      <c r="AS16" t="s">
         <v>420</v>
-      </c>
-      <c r="AF16" t="s">
-        <v>420</v>
-      </c>
-      <c r="AS16" t="s">
-        <v>421</v>
       </c>
     </row>
     <row r="17" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="X17" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="AG17" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="AS17" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
     </row>
     <row r="18" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="C18" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="AS18" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
     </row>
     <row r="19" spans="1:45" x14ac:dyDescent="0.2">
@@ -15827,110 +15839,110 @@
         <v>57</v>
       </c>
       <c r="C19" t="s">
+        <v>419</v>
+      </c>
+      <c r="H19" t="s">
+        <v>419</v>
+      </c>
+      <c r="J19" t="s">
         <v>420</v>
       </c>
-      <c r="H19" t="s">
+      <c r="K19" t="s">
         <v>420</v>
       </c>
-      <c r="J19" t="s">
-        <v>421</v>
-      </c>
-      <c r="K19" t="s">
-        <v>421</v>
-      </c>
       <c r="L19" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="O19" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="P19" t="s">
+        <v>419</v>
+      </c>
+      <c r="Q19" t="s">
         <v>420</v>
       </c>
-      <c r="Q19" t="s">
-        <v>421</v>
-      </c>
       <c r="AC19" t="s">
+        <v>419</v>
+      </c>
+      <c r="AD19" t="s">
+        <v>419</v>
+      </c>
+      <c r="AE19" t="s">
         <v>420</v>
       </c>
-      <c r="AD19" t="s">
+      <c r="AG19" t="s">
+        <v>419</v>
+      </c>
+      <c r="AJ19" t="s">
+        <v>419</v>
+      </c>
+      <c r="AK19" t="s">
+        <v>419</v>
+      </c>
+      <c r="AN19" t="s">
+        <v>419</v>
+      </c>
+      <c r="AQ19" t="s">
+        <v>419</v>
+      </c>
+      <c r="AS19" t="s">
         <v>420</v>
-      </c>
-      <c r="AE19" t="s">
-        <v>421</v>
-      </c>
-      <c r="AG19" t="s">
-        <v>420</v>
-      </c>
-      <c r="AJ19" t="s">
-        <v>420</v>
-      </c>
-      <c r="AK19" t="s">
-        <v>420</v>
-      </c>
-      <c r="AN19" t="s">
-        <v>420</v>
-      </c>
-      <c r="AQ19" t="s">
-        <v>420</v>
-      </c>
-      <c r="AS19" t="s">
-        <v>421</v>
       </c>
     </row>
     <row r="20" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="AA20" t="s">
+        <v>419</v>
+      </c>
+      <c r="AS20" t="s">
         <v>420</v>
-      </c>
-      <c r="AS20" t="s">
-        <v>421</v>
       </c>
     </row>
     <row r="21" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="C21" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="AS21" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
     </row>
     <row r="22" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="X22" t="s">
+        <v>419</v>
+      </c>
+      <c r="AS22" t="s">
         <v>420</v>
-      </c>
-      <c r="AS22" t="s">
-        <v>421</v>
       </c>
     </row>
     <row r="23" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="S23" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="AJ23" t="s">
+        <v>419</v>
+      </c>
+      <c r="AS23" t="s">
         <v>420</v>
-      </c>
-      <c r="AS23" t="s">
-        <v>421</v>
       </c>
     </row>
     <row r="24" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="C24" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
     </row>
   </sheetData>
@@ -18765,493 +18777,620 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:R21"/>
+  <dimension ref="A1:X21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="17.5" style="30" customWidth="1"/>
-    <col min="2" max="2" width="22" style="30" customWidth="1"/>
-    <col min="3" max="3" width="14.33203125" style="30" customWidth="1"/>
-    <col min="4" max="4" width="32.6640625" style="30" customWidth="1"/>
-    <col min="5" max="5" width="18.33203125" style="30" customWidth="1"/>
-    <col min="6" max="6" width="28.33203125" style="30" customWidth="1"/>
-    <col min="7" max="7" width="19" style="30" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="16" style="30" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="22.83203125" style="30" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="23.5" style="30" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="15.5" style="30" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="17.83203125" style="30" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="17.83203125" style="30" customWidth="1"/>
-    <col min="14" max="14" width="21.5" style="30" customWidth="1"/>
-    <col min="15" max="15" width="23" style="30" customWidth="1"/>
-    <col min="16" max="18" width="15.83203125" style="30" customWidth="1"/>
-    <col min="19" max="19" width="8.83203125" style="30" customWidth="1"/>
-    <col min="20" max="16384" width="8.83203125" style="30"/>
+    <col min="2" max="3" width="22" style="30" customWidth="1"/>
+    <col min="4" max="4" width="14.33203125" style="30" customWidth="1"/>
+    <col min="5" max="5" width="32.6640625" style="30" customWidth="1"/>
+    <col min="6" max="6" width="18.33203125" style="30" customWidth="1"/>
+    <col min="7" max="7" width="28.33203125" style="30" customWidth="1"/>
+    <col min="8" max="8" width="19" style="30" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="16" style="30" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="22.83203125" style="30" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="23.5" style="30" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="15.5" style="30" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="17.83203125" style="30" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="17.83203125" style="30" customWidth="1"/>
+    <col min="15" max="20" width="21.5" style="30" customWidth="1"/>
+    <col min="21" max="21" width="23" style="30" customWidth="1"/>
+    <col min="22" max="24" width="15.83203125" style="30" customWidth="1"/>
+    <col min="25" max="25" width="8.83203125" style="30" customWidth="1"/>
+    <col min="26" max="16384" width="8.83203125" style="30"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:24" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="29" t="s">
         <v>190</v>
       </c>
       <c r="B1" s="29"/>
-    </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="C1" s="29"/>
+    </row>
+    <row r="2" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A2" s="31" t="s">
         <v>191</v>
       </c>
       <c r="B2" s="31"/>
-    </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="C2" s="31"/>
+    </row>
+    <row r="3" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A3" s="31"/>
       <c r="B3" s="31"/>
-      <c r="P3" s="19" t="s">
+      <c r="C3" s="31"/>
+      <c r="V3" s="19" t="s">
         <v>73</v>
       </c>
-      <c r="Q3" s="20"/>
-      <c r="R3" s="20"/>
-    </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="W3" s="20"/>
+      <c r="X3" s="20"/>
+    </row>
+    <row r="4" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A4" s="32" t="s">
         <v>57</v>
       </c>
       <c r="B4" s="32" t="s">
         <v>74</v>
       </c>
-      <c r="C4" s="33" t="s">
+      <c r="C4" s="32" t="s">
+        <v>8</v>
+      </c>
+      <c r="D4" s="33" t="s">
         <v>192</v>
       </c>
-      <c r="D4" s="33" t="s">
+      <c r="E4" s="33" t="s">
         <v>21</v>
       </c>
-      <c r="E4" s="33" t="s">
+      <c r="F4" s="33" t="s">
         <v>193</v>
       </c>
-      <c r="F4" s="33" t="s">
+      <c r="G4" s="33" t="s">
         <v>194</v>
       </c>
-      <c r="G4" s="33" t="s">
+      <c r="H4" s="33" t="s">
         <v>195</v>
       </c>
-      <c r="H4" s="33" t="s">
+      <c r="I4" s="33" t="s">
         <v>196</v>
       </c>
-      <c r="I4" s="33" t="s">
+      <c r="J4" s="33" t="s">
         <v>197</v>
       </c>
-      <c r="J4" s="33" t="s">
+      <c r="K4" s="33" t="s">
         <v>198</v>
       </c>
-      <c r="K4" s="33" t="s">
+      <c r="L4" s="33" t="s">
         <v>199</v>
       </c>
-      <c r="L4" s="33" t="s">
+      <c r="M4" s="33" t="s">
         <v>200</v>
       </c>
-      <c r="M4" s="33" t="s">
+      <c r="N4" s="33" t="s">
         <v>201</v>
       </c>
-      <c r="N4" s="33" t="s">
+      <c r="O4" s="33" t="s">
         <v>202</v>
       </c>
-      <c r="O4" s="33" t="s">
+      <c r="P4" s="33" t="s">
+        <v>421</v>
+      </c>
+      <c r="Q4" s="33" t="s">
+        <v>422</v>
+      </c>
+      <c r="R4" s="33" t="s">
+        <v>423</v>
+      </c>
+      <c r="S4" s="33" t="s">
+        <v>242</v>
+      </c>
+      <c r="T4" s="33" t="s">
+        <v>28</v>
+      </c>
+      <c r="U4" s="33" t="s">
         <v>6</v>
       </c>
-      <c r="P4" s="10"/>
-      <c r="Q4" s="10"/>
-      <c r="R4" s="10"/>
-    </row>
-    <row r="5" spans="1:18" ht="34" x14ac:dyDescent="0.2">
+      <c r="V4" s="10"/>
+      <c r="W4" s="10"/>
+      <c r="X4" s="10"/>
+    </row>
+    <row r="5" spans="1:24" ht="34" x14ac:dyDescent="0.2">
       <c r="A5" s="17" t="s">
         <v>59</v>
       </c>
       <c r="B5" s="17"/>
-      <c r="C5" s="15" t="s">
+      <c r="C5" s="17"/>
+      <c r="D5" s="15" t="s">
         <v>203</v>
       </c>
-      <c r="D5" s="15" t="s">
+      <c r="E5" s="15" t="s">
         <v>204</v>
       </c>
-      <c r="E5" s="15"/>
-      <c r="F5" s="15" t="s">
+      <c r="F5" s="15"/>
+      <c r="G5" s="15" t="s">
         <v>205</v>
       </c>
-      <c r="G5" s="15" t="s">
+      <c r="H5" s="15" t="s">
         <v>206</v>
       </c>
-      <c r="H5" s="15">
+      <c r="I5" s="15">
         <v>1</v>
       </c>
-      <c r="I5" s="15"/>
       <c r="J5" s="15"/>
       <c r="K5" s="15"/>
       <c r="L5" s="15"/>
       <c r="M5" s="15"/>
-      <c r="N5" s="17"/>
+      <c r="N5" s="15"/>
       <c r="O5" s="17"/>
-      <c r="P5" s="15"/>
-      <c r="Q5" s="15"/>
-      <c r="R5" s="15"/>
-    </row>
-    <row r="6" spans="1:18" ht="34" x14ac:dyDescent="0.2">
+      <c r="P5" s="17"/>
+      <c r="Q5" s="17"/>
+      <c r="R5" s="17"/>
+      <c r="S5" s="17"/>
+      <c r="T5" s="17"/>
+      <c r="U5" s="17"/>
+      <c r="V5" s="15"/>
+      <c r="W5" s="15"/>
+      <c r="X5" s="15"/>
+    </row>
+    <row r="6" spans="1:24" ht="34" x14ac:dyDescent="0.2">
       <c r="A6" s="17" t="s">
         <v>59</v>
       </c>
       <c r="B6" s="17" t="s">
         <v>157</v>
       </c>
-      <c r="C6" s="15" t="s">
+      <c r="C6" s="17"/>
+      <c r="D6" s="15" t="s">
         <v>122</v>
       </c>
-      <c r="D6" s="15" t="s">
+      <c r="E6" s="15" t="s">
         <v>207</v>
       </c>
-      <c r="E6" s="15"/>
-      <c r="F6" s="27"/>
-      <c r="G6" s="15"/>
+      <c r="F6" s="15"/>
+      <c r="G6" s="27"/>
       <c r="H6" s="15"/>
       <c r="I6" s="15"/>
       <c r="J6" s="15"/>
       <c r="K6" s="15"/>
       <c r="L6" s="15"/>
       <c r="M6" s="15"/>
-      <c r="N6" s="17"/>
+      <c r="N6" s="15"/>
       <c r="O6" s="17"/>
-      <c r="P6" s="15"/>
-      <c r="Q6" s="15"/>
-      <c r="R6" s="15"/>
-    </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="P6" s="17"/>
+      <c r="Q6" s="17"/>
+      <c r="R6" s="17"/>
+      <c r="S6" s="17"/>
+      <c r="T6" s="17"/>
+      <c r="U6" s="17"/>
+      <c r="V6" s="15"/>
+      <c r="W6" s="15"/>
+      <c r="X6" s="15"/>
+    </row>
+    <row r="7" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A7" s="17"/>
       <c r="B7" s="17"/>
-      <c r="C7" s="15"/>
+      <c r="C7" s="17"/>
       <c r="D7" s="15"/>
       <c r="E7" s="15"/>
-      <c r="F7" s="27"/>
-      <c r="G7" s="15"/>
+      <c r="F7" s="15"/>
+      <c r="G7" s="27"/>
       <c r="H7" s="15"/>
       <c r="I7" s="15"/>
       <c r="J7" s="15"/>
       <c r="K7" s="15"/>
       <c r="L7" s="15"/>
       <c r="M7" s="15"/>
-      <c r="N7" s="17"/>
+      <c r="N7" s="15"/>
       <c r="O7" s="17"/>
-      <c r="P7" s="15"/>
-      <c r="Q7" s="15"/>
-      <c r="R7" s="15"/>
-    </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="P7" s="17"/>
+      <c r="Q7" s="17"/>
+      <c r="R7" s="17"/>
+      <c r="S7" s="17"/>
+      <c r="T7" s="17"/>
+      <c r="U7" s="17"/>
+      <c r="V7" s="15"/>
+      <c r="W7" s="15"/>
+      <c r="X7" s="15"/>
+    </row>
+    <row r="8" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A8" s="17"/>
       <c r="B8" s="17"/>
-      <c r="C8" s="15"/>
+      <c r="C8" s="17"/>
       <c r="D8" s="15"/>
       <c r="E8" s="15"/>
-      <c r="F8" s="27"/>
-      <c r="G8" s="15"/>
+      <c r="F8" s="15"/>
+      <c r="G8" s="27"/>
       <c r="H8" s="15"/>
       <c r="I8" s="15"/>
       <c r="J8" s="15"/>
       <c r="K8" s="15"/>
       <c r="L8" s="15"/>
       <c r="M8" s="15"/>
-      <c r="N8" s="17"/>
+      <c r="N8" s="15"/>
       <c r="O8" s="17"/>
-      <c r="P8" s="15"/>
-      <c r="Q8" s="15"/>
-      <c r="R8" s="15"/>
-    </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="P8" s="17"/>
+      <c r="Q8" s="17"/>
+      <c r="R8" s="17"/>
+      <c r="S8" s="17"/>
+      <c r="T8" s="17"/>
+      <c r="U8" s="17"/>
+      <c r="V8" s="15"/>
+      <c r="W8" s="15"/>
+      <c r="X8" s="15"/>
+    </row>
+    <row r="9" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A9" s="17"/>
       <c r="B9" s="17"/>
-      <c r="C9" s="15"/>
+      <c r="C9" s="17"/>
       <c r="D9" s="15"/>
       <c r="E9" s="15"/>
-      <c r="F9" s="27"/>
-      <c r="G9" s="15"/>
+      <c r="F9" s="15"/>
+      <c r="G9" s="27"/>
       <c r="H9" s="15"/>
       <c r="I9" s="15"/>
       <c r="J9" s="15"/>
       <c r="K9" s="15"/>
       <c r="L9" s="15"/>
       <c r="M9" s="15"/>
-      <c r="N9" s="17"/>
+      <c r="N9" s="15"/>
       <c r="O9" s="17"/>
-      <c r="P9" s="15"/>
-      <c r="Q9" s="15"/>
-      <c r="R9" s="15"/>
-    </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="P9" s="17"/>
+      <c r="Q9" s="17"/>
+      <c r="R9" s="17"/>
+      <c r="S9" s="17"/>
+      <c r="T9" s="17"/>
+      <c r="U9" s="17"/>
+      <c r="V9" s="15"/>
+      <c r="W9" s="15"/>
+      <c r="X9" s="15"/>
+    </row>
+    <row r="10" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A10" s="17"/>
       <c r="B10" s="17"/>
-      <c r="C10" s="15"/>
+      <c r="C10" s="17"/>
       <c r="D10" s="15"/>
       <c r="E10" s="15"/>
-      <c r="F10" s="27"/>
-      <c r="G10" s="15"/>
+      <c r="F10" s="15"/>
+      <c r="G10" s="27"/>
       <c r="H10" s="15"/>
       <c r="I10" s="15"/>
       <c r="J10" s="15"/>
       <c r="K10" s="15"/>
       <c r="L10" s="15"/>
       <c r="M10" s="15"/>
-      <c r="N10" s="17"/>
+      <c r="N10" s="15"/>
       <c r="O10" s="17"/>
-      <c r="P10" s="15"/>
-      <c r="Q10" s="15"/>
-      <c r="R10" s="15"/>
-    </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="P10" s="17"/>
+      <c r="Q10" s="17"/>
+      <c r="R10" s="17"/>
+      <c r="S10" s="17"/>
+      <c r="T10" s="17"/>
+      <c r="U10" s="17"/>
+      <c r="V10" s="15"/>
+      <c r="W10" s="15"/>
+      <c r="X10" s="15"/>
+    </row>
+    <row r="11" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A11" s="17"/>
       <c r="B11" s="17"/>
-      <c r="C11" s="15"/>
+      <c r="C11" s="17"/>
       <c r="D11" s="15"/>
       <c r="E11" s="15"/>
-      <c r="F11" s="27"/>
-      <c r="G11" s="15"/>
+      <c r="F11" s="15"/>
+      <c r="G11" s="27"/>
       <c r="H11" s="15"/>
       <c r="I11" s="15"/>
       <c r="J11" s="15"/>
       <c r="K11" s="15"/>
       <c r="L11" s="15"/>
       <c r="M11" s="15"/>
-      <c r="N11" s="17"/>
+      <c r="N11" s="15"/>
       <c r="O11" s="17"/>
-      <c r="P11" s="15"/>
-      <c r="Q11" s="15"/>
-      <c r="R11" s="15"/>
-    </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="P11" s="17"/>
+      <c r="Q11" s="17"/>
+      <c r="R11" s="17"/>
+      <c r="S11" s="17"/>
+      <c r="T11" s="17"/>
+      <c r="U11" s="17"/>
+      <c r="V11" s="15"/>
+      <c r="W11" s="15"/>
+      <c r="X11" s="15"/>
+    </row>
+    <row r="12" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A12" s="17"/>
       <c r="B12" s="17"/>
-      <c r="C12" s="15"/>
+      <c r="C12" s="17"/>
       <c r="D12" s="15"/>
       <c r="E12" s="15"/>
-      <c r="F12" s="27"/>
-      <c r="G12" s="15"/>
+      <c r="F12" s="15"/>
+      <c r="G12" s="27"/>
       <c r="H12" s="15"/>
       <c r="I12" s="15"/>
       <c r="J12" s="15"/>
       <c r="K12" s="15"/>
       <c r="L12" s="15"/>
       <c r="M12" s="15"/>
-      <c r="N12" s="17"/>
+      <c r="N12" s="15"/>
       <c r="O12" s="17"/>
-      <c r="P12" s="15"/>
-      <c r="Q12" s="15"/>
-      <c r="R12" s="15"/>
-    </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="P12" s="17"/>
+      <c r="Q12" s="17"/>
+      <c r="R12" s="17"/>
+      <c r="S12" s="17"/>
+      <c r="T12" s="17"/>
+      <c r="U12" s="17"/>
+      <c r="V12" s="15"/>
+      <c r="W12" s="15"/>
+      <c r="X12" s="15"/>
+    </row>
+    <row r="13" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A13" s="17"/>
       <c r="B13" s="17"/>
-      <c r="C13" s="15"/>
+      <c r="C13" s="17"/>
       <c r="D13" s="15"/>
       <c r="E13" s="15"/>
-      <c r="F13" s="27"/>
-      <c r="G13" s="15"/>
+      <c r="F13" s="15"/>
+      <c r="G13" s="27"/>
       <c r="H13" s="15"/>
       <c r="I13" s="15"/>
       <c r="J13" s="15"/>
       <c r="K13" s="15"/>
       <c r="L13" s="15"/>
       <c r="M13" s="15"/>
-      <c r="N13" s="17"/>
+      <c r="N13" s="15"/>
       <c r="O13" s="17"/>
-      <c r="P13" s="15"/>
-      <c r="Q13" s="15"/>
-      <c r="R13" s="15"/>
-    </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="P13" s="17"/>
+      <c r="Q13" s="17"/>
+      <c r="R13" s="17"/>
+      <c r="S13" s="17"/>
+      <c r="T13" s="17"/>
+      <c r="U13" s="17"/>
+      <c r="V13" s="15"/>
+      <c r="W13" s="15"/>
+      <c r="X13" s="15"/>
+    </row>
+    <row r="14" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A14" s="17"/>
       <c r="B14" s="17"/>
-      <c r="C14" s="15"/>
+      <c r="C14" s="17"/>
       <c r="D14" s="15"/>
       <c r="E14" s="15"/>
-      <c r="F14" s="27"/>
-      <c r="G14" s="15"/>
+      <c r="F14" s="15"/>
+      <c r="G14" s="27"/>
       <c r="H14" s="15"/>
       <c r="I14" s="15"/>
       <c r="J14" s="15"/>
       <c r="K14" s="15"/>
       <c r="L14" s="15"/>
       <c r="M14" s="15"/>
-      <c r="N14" s="17"/>
+      <c r="N14" s="15"/>
       <c r="O14" s="17"/>
-      <c r="P14" s="15"/>
-      <c r="Q14" s="15"/>
-      <c r="R14" s="15"/>
-    </row>
-    <row r="15" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="P14" s="17"/>
+      <c r="Q14" s="17"/>
+      <c r="R14" s="17"/>
+      <c r="S14" s="17"/>
+      <c r="T14" s="17"/>
+      <c r="U14" s="17"/>
+      <c r="V14" s="15"/>
+      <c r="W14" s="15"/>
+      <c r="X14" s="15"/>
+    </row>
+    <row r="15" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A15" s="17"/>
       <c r="B15" s="17"/>
-      <c r="C15" s="15"/>
+      <c r="C15" s="17"/>
       <c r="D15" s="15"/>
       <c r="E15" s="15"/>
-      <c r="F15" s="27"/>
-      <c r="G15" s="15"/>
+      <c r="F15" s="15"/>
+      <c r="G15" s="27"/>
       <c r="H15" s="15"/>
       <c r="I15" s="15"/>
       <c r="J15" s="15"/>
       <c r="K15" s="15"/>
       <c r="L15" s="15"/>
       <c r="M15" s="15"/>
-      <c r="N15" s="17"/>
+      <c r="N15" s="15"/>
       <c r="O15" s="17"/>
-      <c r="P15" s="15"/>
-      <c r="Q15" s="15"/>
-      <c r="R15" s="15"/>
-    </row>
-    <row r="16" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="P15" s="17"/>
+      <c r="Q15" s="17"/>
+      <c r="R15" s="17"/>
+      <c r="S15" s="17"/>
+      <c r="T15" s="17"/>
+      <c r="U15" s="17"/>
+      <c r="V15" s="15"/>
+      <c r="W15" s="15"/>
+      <c r="X15" s="15"/>
+    </row>
+    <row r="16" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A16" s="17"/>
       <c r="B16" s="17"/>
-      <c r="C16" s="15"/>
+      <c r="C16" s="17"/>
       <c r="D16" s="15"/>
       <c r="E16" s="15"/>
-      <c r="F16" s="27"/>
-      <c r="G16" s="15"/>
+      <c r="F16" s="15"/>
+      <c r="G16" s="27"/>
       <c r="H16" s="15"/>
       <c r="I16" s="15"/>
       <c r="J16" s="15"/>
       <c r="K16" s="15"/>
       <c r="L16" s="15"/>
       <c r="M16" s="15"/>
-      <c r="N16" s="17"/>
+      <c r="N16" s="15"/>
       <c r="O16" s="17"/>
-      <c r="P16" s="15"/>
-      <c r="Q16" s="15"/>
-      <c r="R16" s="15"/>
-    </row>
-    <row r="17" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="P16" s="17"/>
+      <c r="Q16" s="17"/>
+      <c r="R16" s="17"/>
+      <c r="S16" s="17"/>
+      <c r="T16" s="17"/>
+      <c r="U16" s="17"/>
+      <c r="V16" s="15"/>
+      <c r="W16" s="15"/>
+      <c r="X16" s="15"/>
+    </row>
+    <row r="17" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A17" s="17"/>
       <c r="B17" s="17"/>
-      <c r="C17" s="15"/>
+      <c r="C17" s="17"/>
       <c r="D17" s="15"/>
       <c r="E17" s="15"/>
-      <c r="F17" s="27"/>
-      <c r="G17" s="15"/>
+      <c r="F17" s="15"/>
+      <c r="G17" s="27"/>
       <c r="H17" s="15"/>
       <c r="I17" s="15"/>
       <c r="J17" s="15"/>
       <c r="K17" s="15"/>
       <c r="L17" s="15"/>
       <c r="M17" s="15"/>
-      <c r="N17" s="17"/>
+      <c r="N17" s="15"/>
       <c r="O17" s="17"/>
-      <c r="P17" s="15"/>
-      <c r="Q17" s="15"/>
-      <c r="R17" s="15"/>
-    </row>
-    <row r="18" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="P17" s="17"/>
+      <c r="Q17" s="17"/>
+      <c r="R17" s="17"/>
+      <c r="S17" s="17"/>
+      <c r="T17" s="17"/>
+      <c r="U17" s="17"/>
+      <c r="V17" s="15"/>
+      <c r="W17" s="15"/>
+      <c r="X17" s="15"/>
+    </row>
+    <row r="18" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A18" s="17"/>
       <c r="B18" s="17"/>
-      <c r="C18" s="15"/>
+      <c r="C18" s="17"/>
       <c r="D18" s="15"/>
       <c r="E18" s="15"/>
-      <c r="F18" s="27"/>
-      <c r="G18" s="15"/>
+      <c r="F18" s="15"/>
+      <c r="G18" s="27"/>
       <c r="H18" s="15"/>
       <c r="I18" s="15"/>
       <c r="J18" s="15"/>
       <c r="K18" s="15"/>
       <c r="L18" s="15"/>
       <c r="M18" s="15"/>
-      <c r="N18" s="17"/>
+      <c r="N18" s="15"/>
       <c r="O18" s="17"/>
-      <c r="P18" s="15"/>
-      <c r="Q18" s="15"/>
-      <c r="R18" s="15"/>
-    </row>
-    <row r="19" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="P18" s="17"/>
+      <c r="Q18" s="17"/>
+      <c r="R18" s="17"/>
+      <c r="S18" s="17"/>
+      <c r="T18" s="17"/>
+      <c r="U18" s="17"/>
+      <c r="V18" s="15"/>
+      <c r="W18" s="15"/>
+      <c r="X18" s="15"/>
+    </row>
+    <row r="19" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A19" s="17"/>
       <c r="B19" s="17"/>
-      <c r="C19" s="15"/>
+      <c r="C19" s="17"/>
       <c r="D19" s="15"/>
       <c r="E19" s="15"/>
-      <c r="F19" s="27"/>
-      <c r="G19" s="15"/>
+      <c r="F19" s="15"/>
+      <c r="G19" s="27"/>
       <c r="H19" s="15"/>
       <c r="I19" s="15"/>
       <c r="J19" s="15"/>
       <c r="K19" s="15"/>
       <c r="L19" s="15"/>
       <c r="M19" s="15"/>
-      <c r="N19" s="17"/>
+      <c r="N19" s="15"/>
       <c r="O19" s="17"/>
-      <c r="P19" s="15"/>
-      <c r="Q19" s="15"/>
-      <c r="R19" s="15"/>
-    </row>
-    <row r="20" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="P19" s="17"/>
+      <c r="Q19" s="17"/>
+      <c r="R19" s="17"/>
+      <c r="S19" s="17"/>
+      <c r="T19" s="17"/>
+      <c r="U19" s="17"/>
+      <c r="V19" s="15"/>
+      <c r="W19" s="15"/>
+      <c r="X19" s="15"/>
+    </row>
+    <row r="20" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A20" s="17"/>
       <c r="B20" s="17"/>
-      <c r="C20" s="15"/>
+      <c r="C20" s="17"/>
       <c r="D20" s="15"/>
       <c r="E20" s="15"/>
-      <c r="F20" s="27"/>
-      <c r="G20" s="15"/>
+      <c r="F20" s="15"/>
+      <c r="G20" s="27"/>
       <c r="H20" s="15"/>
       <c r="I20" s="15"/>
       <c r="J20" s="15"/>
       <c r="K20" s="15"/>
       <c r="L20" s="15"/>
       <c r="M20" s="15"/>
-      <c r="N20" s="17"/>
+      <c r="N20" s="15"/>
       <c r="O20" s="17"/>
-      <c r="P20" s="15"/>
-      <c r="Q20" s="15"/>
-      <c r="R20" s="15"/>
-    </row>
-    <row r="21" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="P20" s="17"/>
+      <c r="Q20" s="17"/>
+      <c r="R20" s="17"/>
+      <c r="S20" s="17"/>
+      <c r="T20" s="17"/>
+      <c r="U20" s="17"/>
+      <c r="V20" s="15"/>
+      <c r="W20" s="15"/>
+      <c r="X20" s="15"/>
+    </row>
+    <row r="21" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A21" s="17"/>
       <c r="B21" s="17"/>
-      <c r="C21" s="15"/>
+      <c r="C21" s="17"/>
       <c r="D21" s="15"/>
       <c r="E21" s="15"/>
-      <c r="F21" s="27"/>
-      <c r="G21" s="15"/>
+      <c r="F21" s="15"/>
+      <c r="G21" s="27"/>
       <c r="H21" s="15"/>
       <c r="I21" s="15"/>
       <c r="J21" s="15"/>
       <c r="K21" s="15"/>
       <c r="L21" s="15"/>
       <c r="M21" s="15"/>
-      <c r="N21" s="17"/>
+      <c r="N21" s="15"/>
       <c r="O21" s="17"/>
-      <c r="P21" s="15"/>
-      <c r="Q21" s="15"/>
-      <c r="R21" s="15"/>
+      <c r="P21" s="17"/>
+      <c r="Q21" s="17"/>
+      <c r="R21" s="17"/>
+      <c r="S21" s="17"/>
+      <c r="T21" s="17"/>
+      <c r="U21" s="17"/>
+      <c r="V21" s="15"/>
+      <c r="W21" s="15"/>
+      <c r="X21" s="15"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="E5:E21">
+  <conditionalFormatting sqref="F5:F21">
     <cfRule type="expression" dxfId="7" priority="1" stopIfTrue="1">
-      <formula>C5="sql"</formula>
+      <formula>D5="sql"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F5:F21">
+  <conditionalFormatting sqref="G5:G21">
     <cfRule type="expression" dxfId="6" priority="2" stopIfTrue="1">
-      <formula>C5="library"</formula>
+      <formula>D5="library"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="15">
-    <dataValidation allowBlank="1" sqref="C22:G42 P5:R21" xr:uid="{00000000-0002-0000-0400-000000000000}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Data Quality Type" prompt="Data quality rules support different levels/stages of data quality attributes:_x000a__x000a_Text: A human-readable text that describes the quality of the data._x000a_Library rules: A maintained library of commonly-used predefined quality attributes such as rowCount, unique" sqref="C4" xr:uid="{00000000-0002-0000-0400-000001000000}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Quality Scheduler" prompt="Name of the scheduler that runs the quality check, such as cron, Airflow, or Github Action." sqref="L5:M21" xr:uid="{00000000-0002-0000-0400-000002000000}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Quality Severity" prompt="The severity of the data quality rule, such as error or warning." sqref="K5:K21" xr:uid="{00000000-0002-0000-0400-000003000000}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Quality Implementation" prompt="The data quality check in the engine's specific format." sqref="J5:J21" xr:uid="{00000000-0002-0000-0400-000004000000}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Quality Engine" prompt="Required for custom DQ rule: name of the third-party engine being used. Any value is authorized here but common values are soda, greatExpectations, montecarlo, etc." sqref="I5:I21" xr:uid="{00000000-0002-0000-0400-000005000000}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Quality Threshold Value" prompt="The acutal value for the treshold operator._x000a_For mustBeBetween adn mustNotBeBetween, use [lowerBoundry, upperBoundy] syntax, e.g. [0, 100]." sqref="H5:H21" xr:uid="{00000000-0002-0000-0400-000006000000}"/>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Quality Operator" prompt="The comparation operator specifies the condition to validate the rule._x000a_Use it together with the threshold value, e.g. mustBe 0, or mustBeBetween [0,100]_x000a_This is applicable for quality type sql and some library rules." sqref="G5:G21" xr:uid="{00000000-0002-0000-0400-000007000000}">
+  <dataValidations count="17">
+    <dataValidation allowBlank="1" sqref="D22:H42 V5:X21" xr:uid="{00000000-0002-0000-0400-000000000000}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Data Quality Type" prompt="Data quality rules support different levels/stages of data quality attributes:_x000a__x000a_Text: A human-readable text that describes the quality of the data._x000a_Library rules: A maintained library of commonly-used predefined quality attributes such as rowCount, unique" sqref="D4" xr:uid="{00000000-0002-0000-0400-000001000000}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Quality Scheduler" prompt="Name of the scheduler that runs the quality check, such as cron, Airflow, or Github Action." sqref="M5:N21" xr:uid="{00000000-0002-0000-0400-000002000000}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Quality Severity" prompt="The severity of the data quality rule, such as error or warning." sqref="L5:L21" xr:uid="{00000000-0002-0000-0400-000003000000}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Quality Implementation" prompt="The data quality check in the engine's specific format." sqref="K5:K21" xr:uid="{00000000-0002-0000-0400-000004000000}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Quality Engine" prompt="Required for custom DQ rule: name of the third-party engine being used. Any value is authorized here but common values are soda, greatExpectations, montecarlo, etc." sqref="J5:J21" xr:uid="{00000000-0002-0000-0400-000005000000}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Quality Threshold Value" prompt="The acutal value for the treshold operator._x000a_For mustBeBetween adn mustNotBeBetween, use [lowerBoundry, upperBoundy] syntax, e.g. [0, 100]." sqref="I5:I21" xr:uid="{00000000-0002-0000-0400-000006000000}"/>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Quality Operator" prompt="The comparation operator specifies the condition to validate the rule._x000a_Use it together with the threshold value, e.g. mustBe 0, or mustBeBetween [0,100]_x000a_This is applicable for quality type sql and some library rules." sqref="H5:H21" xr:uid="{00000000-0002-0000-0400-000007000000}">
       <formula1>"mustBe, mustNotBe, mustBeGreaterThan, mustBeGreaterOrEqualTo, mustBeLessThan, mustBeLessOrEqualTo, mustBeBetween, mustNotBeBetween"</formula1>
     </dataValidation>
-    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Quality Query" prompt="A single SQL query that returns either a numeric or boolean value for comparison. The query must be written in the SQL dialect specific to the provided server. " sqref="F5:F21" xr:uid="{00000000-0002-0000-0400-000008000000}"/>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Quality Metric" prompt="The expected or guaranteed data quality from a business perspective._x000a__x000a_Maps to quality.description" sqref="E5:E21" xr:uid="{00000000-0002-0000-0400-000009000000}">
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Quality Query" prompt="A single SQL query that returns either a numeric or boolean value for comparison. The query must be written in the SQL dialect specific to the provided server. " sqref="G5:G21" xr:uid="{00000000-0002-0000-0400-000008000000}"/>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Quality Metric" prompt="The expected or guaranteed data quality from a business perspective._x000a__x000a_Maps to quality.description" sqref="F5:F21" xr:uid="{00000000-0002-0000-0400-000009000000}">
       <formula1>"nullValues,missingValues,invalidValues,duplicateValues,rowCount"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="C5:C21" xr:uid="{00000000-0002-0000-0400-00000A000000}">
+    <dataValidation type="list" allowBlank="1" sqref="D5:D21" xr:uid="{00000000-0002-0000-0400-00000A000000}">
       <formula1>"text,library,sql,custom"</formula1>
     </dataValidation>
-    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Quality" prompt="The expected or guaranteed data quality from a business perspective._x000a__x000a_Maps to quality.description" sqref="D5:D21" xr:uid="{00000000-0002-0000-0400-00000B000000}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Quality" prompt="The expected or guaranteed data quality from a business perspective._x000a__x000a_Maps to quality.description" sqref="E5:E21" xr:uid="{00000000-0002-0000-0400-00000B000000}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Schema" prompt="The schema name must match the name of the schema (table, ...) in the previous sheets." sqref="A4" xr:uid="{00000000-0002-0000-0400-00000C000000}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Property" prompt="Optional: Leave empty, if this is a schema-level quality check._x000a_The property must match the property name in the schema._x000a_" sqref="B4" xr:uid="{00000000-0002-0000-0400-00000D000000}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Rule" prompt="The predefined data quality rule from the library._x000a_Only appliable if &quot;Quality Type&quot; is set to &quot;library&quot; or empty (which is library by default, if a rule is defined)" sqref="E4" xr:uid="{00000000-0002-0000-0400-00000E000000}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Rule" prompt="The predefined data quality rule from the library._x000a_Only appliable if &quot;Quality Type&quot; is set to &quot;library&quot; or empty (which is library by default, if a rule is defined)" sqref="F4" xr:uid="{00000000-0002-0000-0400-00000E000000}"/>
+    <dataValidation allowBlank="1" showErrorMessage="1" promptTitle="Property" prompt="Optional: Leave empty, if this is a schema-level quality check._x000a_The property must match the property name in the schema._x000a_" sqref="C4" xr:uid="{9F023347-9DDC-434C-8107-9602E4047228}"/>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="P5:P100" xr:uid="{64939BE5-C5FF-1C47-9DBB-3E91F07497C9}">
+      <formula1>"accuracy,completeness,conformity,consistency,coverage,timeliness,uniqueness"</formula1>
+    </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
@@ -19870,250 +20009,294 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:K21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="33.1640625" style="2" customWidth="1"/>
-    <col min="2" max="2" width="59.6640625" style="2" customWidth="1"/>
-    <col min="3" max="3" width="39.33203125" style="2" customWidth="1"/>
-    <col min="4" max="4" width="32.83203125" style="2" customWidth="1"/>
-    <col min="5" max="5" width="34.6640625" style="2" customWidth="1"/>
-    <col min="6" max="6" width="26.1640625" style="2" customWidth="1"/>
-    <col min="7" max="9" width="15.83203125" style="2" customWidth="1"/>
-    <col min="10" max="10" width="8.83203125" style="2" customWidth="1"/>
-    <col min="11" max="16384" width="8.83203125" style="2"/>
+    <col min="1" max="2" width="16.83203125" style="2" customWidth="1"/>
+    <col min="3" max="3" width="33.1640625" style="2" customWidth="1"/>
+    <col min="4" max="4" width="59.6640625" style="2" customWidth="1"/>
+    <col min="5" max="5" width="39.33203125" style="2" customWidth="1"/>
+    <col min="6" max="6" width="32.83203125" style="2" customWidth="1"/>
+    <col min="7" max="7" width="34.6640625" style="2" customWidth="1"/>
+    <col min="8" max="8" width="26.1640625" style="2" customWidth="1"/>
+    <col min="9" max="11" width="15.83203125" style="2" customWidth="1"/>
+    <col min="12" max="12" width="8.83203125" style="2" customWidth="1"/>
+    <col min="13" max="16384" width="8.83203125" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>233</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A2" s="4" t="s">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A2" s="39" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="I3" s="19" t="s">
+        <v>73</v>
+      </c>
+      <c r="J3" s="20"/>
+      <c r="K3" s="20"/>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A4" s="9" t="s">
+        <v>213</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>425</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>223</v>
+      </c>
+      <c r="D4" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="E4" s="10" t="s">
         <v>234</v>
       </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="G3" s="19" t="s">
-        <v>73</v>
-      </c>
-      <c r="H3" s="20"/>
-      <c r="I3" s="20"/>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A4" s="9" t="s">
-        <v>223</v>
-      </c>
-      <c r="B4" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="C4" s="10" t="s">
+      <c r="F4" s="10" t="s">
         <v>235</v>
       </c>
-      <c r="D4" s="10" t="s">
+      <c r="G4" s="10" t="s">
         <v>236</v>
       </c>
-      <c r="E4" s="10" t="s">
-        <v>237</v>
-      </c>
-      <c r="F4" s="10" t="s">
+      <c r="H4" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="G4" s="10"/>
-      <c r="H4" s="10"/>
       <c r="I4" s="10"/>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J4" s="10"/>
+      <c r="K4" s="10"/>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A5" s="5"/>
       <c r="B5" s="5"/>
       <c r="C5" s="5"/>
       <c r="D5" s="5"/>
       <c r="E5" s="5"/>
       <c r="F5" s="5"/>
-      <c r="G5" s="15"/>
-      <c r="H5" s="15"/>
+      <c r="G5" s="5"/>
+      <c r="H5" s="5"/>
       <c r="I5" s="15"/>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J5" s="15"/>
+      <c r="K5" s="15"/>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A6" s="5"/>
       <c r="B6" s="5"/>
       <c r="C6" s="5"/>
       <c r="D6" s="5"/>
       <c r="E6" s="5"/>
       <c r="F6" s="5"/>
-      <c r="G6" s="15"/>
-      <c r="H6" s="15"/>
+      <c r="G6" s="5"/>
+      <c r="H6" s="5"/>
       <c r="I6" s="15"/>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J6" s="15"/>
+      <c r="K6" s="15"/>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A7" s="5"/>
       <c r="B7" s="5"/>
       <c r="C7" s="5"/>
       <c r="D7" s="5"/>
       <c r="E7" s="5"/>
       <c r="F7" s="5"/>
-      <c r="G7" s="15"/>
-      <c r="H7" s="15"/>
+      <c r="G7" s="5"/>
+      <c r="H7" s="5"/>
       <c r="I7" s="15"/>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J7" s="15"/>
+      <c r="K7" s="15"/>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A8" s="5"/>
       <c r="B8" s="5"/>
       <c r="C8" s="5"/>
       <c r="D8" s="5"/>
       <c r="E8" s="5"/>
       <c r="F8" s="5"/>
-      <c r="G8" s="15"/>
-      <c r="H8" s="15"/>
+      <c r="G8" s="5"/>
+      <c r="H8" s="5"/>
       <c r="I8" s="15"/>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J8" s="15"/>
+      <c r="K8" s="15"/>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A9" s="5"/>
       <c r="B9" s="5"/>
       <c r="C9" s="5"/>
       <c r="D9" s="5"/>
       <c r="E9" s="5"/>
       <c r="F9" s="5"/>
-      <c r="G9" s="15"/>
-      <c r="H9" s="15"/>
+      <c r="G9" s="5"/>
+      <c r="H9" s="5"/>
       <c r="I9" s="15"/>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J9" s="15"/>
+      <c r="K9" s="15"/>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A10" s="5"/>
       <c r="B10" s="5"/>
       <c r="C10" s="5"/>
       <c r="D10" s="5"/>
       <c r="E10" s="5"/>
       <c r="F10" s="5"/>
-      <c r="G10" s="15"/>
-      <c r="H10" s="15"/>
+      <c r="G10" s="5"/>
+      <c r="H10" s="5"/>
       <c r="I10" s="15"/>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J10" s="15"/>
+      <c r="K10" s="15"/>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A11" s="5"/>
       <c r="B11" s="5"/>
       <c r="C11" s="5"/>
       <c r="D11" s="5"/>
       <c r="E11" s="5"/>
       <c r="F11" s="5"/>
-      <c r="G11" s="15"/>
-      <c r="H11" s="15"/>
+      <c r="G11" s="5"/>
+      <c r="H11" s="5"/>
       <c r="I11" s="15"/>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J11" s="15"/>
+      <c r="K11" s="15"/>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A12" s="5"/>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
       <c r="D12" s="5"/>
       <c r="E12" s="5"/>
       <c r="F12" s="5"/>
-      <c r="G12" s="15"/>
-      <c r="H12" s="15"/>
+      <c r="G12" s="5"/>
+      <c r="H12" s="5"/>
       <c r="I12" s="15"/>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J12" s="15"/>
+      <c r="K12" s="15"/>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A13" s="5"/>
       <c r="B13" s="5"/>
       <c r="C13" s="5"/>
       <c r="D13" s="5"/>
       <c r="E13" s="5"/>
       <c r="F13" s="5"/>
-      <c r="G13" s="15"/>
-      <c r="H13" s="15"/>
+      <c r="G13" s="5"/>
+      <c r="H13" s="5"/>
       <c r="I13" s="15"/>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J13" s="15"/>
+      <c r="K13" s="15"/>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A14" s="5"/>
       <c r="B14" s="5"/>
       <c r="C14" s="5"/>
       <c r="D14" s="5"/>
       <c r="E14" s="5"/>
       <c r="F14" s="5"/>
-      <c r="G14" s="15"/>
-      <c r="H14" s="15"/>
+      <c r="G14" s="5"/>
+      <c r="H14" s="5"/>
       <c r="I14" s="15"/>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J14" s="15"/>
+      <c r="K14" s="15"/>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A15" s="5"/>
       <c r="B15" s="5"/>
       <c r="C15" s="5"/>
       <c r="D15" s="5"/>
       <c r="E15" s="5"/>
       <c r="F15" s="5"/>
-      <c r="G15" s="15"/>
-      <c r="H15" s="15"/>
+      <c r="G15" s="5"/>
+      <c r="H15" s="5"/>
       <c r="I15" s="15"/>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J15" s="15"/>
+      <c r="K15" s="15"/>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A16" s="5"/>
       <c r="B16" s="5"/>
       <c r="C16" s="5"/>
       <c r="D16" s="5"/>
       <c r="E16" s="5"/>
       <c r="F16" s="5"/>
-      <c r="G16" s="15"/>
-      <c r="H16" s="15"/>
+      <c r="G16" s="5"/>
+      <c r="H16" s="5"/>
       <c r="I16" s="15"/>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J16" s="15"/>
+      <c r="K16" s="15"/>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A17" s="5"/>
       <c r="B17" s="5"/>
       <c r="C17" s="5"/>
       <c r="D17" s="5"/>
       <c r="E17" s="5"/>
       <c r="F17" s="5"/>
-      <c r="G17" s="15"/>
-      <c r="H17" s="15"/>
+      <c r="G17" s="5"/>
+      <c r="H17" s="5"/>
       <c r="I17" s="15"/>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J17" s="15"/>
+      <c r="K17" s="15"/>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A18" s="5"/>
       <c r="B18" s="5"/>
       <c r="C18" s="5"/>
       <c r="D18" s="5"/>
       <c r="E18" s="5"/>
       <c r="F18" s="5"/>
-      <c r="G18" s="15"/>
-      <c r="H18" s="15"/>
+      <c r="G18" s="5"/>
+      <c r="H18" s="5"/>
       <c r="I18" s="15"/>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J18" s="15"/>
+      <c r="K18" s="15"/>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A19" s="5"/>
       <c r="B19" s="5"/>
       <c r="C19" s="5"/>
       <c r="D19" s="5"/>
       <c r="E19" s="5"/>
       <c r="F19" s="5"/>
-      <c r="G19" s="15"/>
-      <c r="H19" s="15"/>
+      <c r="G19" s="5"/>
+      <c r="H19" s="5"/>
       <c r="I19" s="15"/>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J19" s="15"/>
+      <c r="K19" s="15"/>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A20" s="5"/>
       <c r="B20" s="5"/>
       <c r="C20" s="5"/>
       <c r="D20" s="5"/>
       <c r="E20" s="5"/>
       <c r="F20" s="5"/>
-      <c r="G20" s="15"/>
-      <c r="H20" s="15"/>
+      <c r="G20" s="5"/>
+      <c r="H20" s="5"/>
       <c r="I20" s="15"/>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J20" s="15"/>
+      <c r="K20" s="15"/>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A21" s="5"/>
       <c r="B21" s="5"/>
       <c r="C21" s="5"/>
       <c r="D21" s="5"/>
       <c r="E21" s="5"/>
       <c r="F21" s="5"/>
-      <c r="G21" s="15"/>
-      <c r="H21" s="15"/>
+      <c r="G21" s="5"/>
+      <c r="H21" s="5"/>
       <c r="I21" s="15"/>
+      <c r="J21" s="15"/>
+      <c r="K21" s="15"/>
     </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation allowBlank="1" sqref="B5:E61 F5:I21" xr:uid="{00000000-0002-0000-0700-000000000000}"/>
+  <dataValidations count="2">
+    <dataValidation allowBlank="1" sqref="D5:G61 H5:K21" xr:uid="{00000000-0002-0000-0700-000000000000}"/>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A5:A100" xr:uid="{6D92BFAD-5F8B-FB42-AB19-4A54367F4906}">
+      <formula1>"Contract,Server"</formula1>
+    </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -20140,12 +20323,12 @@
   <sheetData>
     <row r="1" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.2">
@@ -20153,7 +20336,7 @@
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A4" s="7" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="B4" s="26"/>
     </row>
@@ -20169,19 +20352,19 @@
         <v>74</v>
       </c>
       <c r="B6" s="10" t="s">
+        <v>240</v>
+      </c>
+      <c r="C6" s="10" t="s">
         <v>241</v>
       </c>
-      <c r="C6" s="10" t="s">
+      <c r="D6" s="10" t="s">
         <v>242</v>
       </c>
-      <c r="D6" s="10" t="s">
+      <c r="E6" s="10" t="s">
         <v>243</v>
       </c>
-      <c r="E6" s="10" t="s">
+      <c r="F6" s="10" t="s">
         <v>244</v>
-      </c>
-      <c r="F6" s="10" t="s">
-        <v>245</v>
       </c>
       <c r="G6" s="10" t="s">
         <v>21</v>
@@ -20201,18 +20384,18 @@
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A7" s="5" t="s">
+        <v>245</v>
+      </c>
+      <c r="B7" s="5" t="s">
         <v>246</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>247</v>
       </c>
       <c r="C7" s="5"/>
       <c r="D7" s="5" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="E7" s="5"/>
       <c r="F7" s="5" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="G7" s="5"/>
       <c r="H7" s="5"/>

</xml_diff>

<commit_message>
fix schema logical type field in example
</commit_message>
<xml_diff>
--- a/examples/shipments-odcs.xlsx
+++ b/examples/shipments-odcs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jakob/entropyData/open-data-contract-standard-excel-template/examples/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F86B5D8-5546-0043-AD7D-BF6A6DC88DCF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EB5EC1E-CE53-6B4B-9783-B7C51AD4DE7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="780" windowWidth="34200" windowHeight="21460" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -61,17 +61,17 @@
     <definedName name="quality">Quality!$A$4:$BF$300</definedName>
     <definedName name="relationships">Relationships!$A$4:$AZ$300</definedName>
     <definedName name="roles" localSheetId="7">Roles!$A$4:$AZ$1000</definedName>
-    <definedName name="schema.businessName" localSheetId="2">'Schema shipments'!$B$10</definedName>
-    <definedName name="schema.context.instructions" localSheetId="2">'Schema shipments'!$B$15</definedName>
-    <definedName name="schema.dataGranularityDescription" localSheetId="2">'Schema shipments'!$B$12</definedName>
-    <definedName name="schema.deprecated" localSheetId="2">'Schema shipments'!$B$16</definedName>
-    <definedName name="schema.description" localSheetId="2">'Schema shipments'!$B$9</definedName>
-    <definedName name="schema.id" localSheetId="2">'Schema shipments'!$B$14</definedName>
+    <definedName name="schema.businessName" localSheetId="2">'Schema shipments'!$B$9</definedName>
+    <definedName name="schema.context.instructions" localSheetId="2">'Schema shipments'!$B$14</definedName>
+    <definedName name="schema.dataGranularityDescription" localSheetId="2">'Schema shipments'!$B$11</definedName>
+    <definedName name="schema.deprecated" localSheetId="2">'Schema shipments'!$B$15</definedName>
+    <definedName name="schema.description" localSheetId="2">'Schema shipments'!$B$8</definedName>
+    <definedName name="schema.id" localSheetId="2">'Schema shipments'!$B$13</definedName>
     <definedName name="schema.name" localSheetId="2">'Schema shipments'!$B$5</definedName>
-    <definedName name="schema.physicalName" localSheetId="2">'Schema shipments'!$B$11</definedName>
-    <definedName name="schema.physicalType" localSheetId="2">'Schema shipments'!$B$7</definedName>
-    <definedName name="schema.properties" localSheetId="2">'Schema shipments'!$A$18:$AW$986</definedName>
-    <definedName name="schema.tags" localSheetId="2">'Schema shipments'!$B$13</definedName>
+    <definedName name="schema.physicalName" localSheetId="2">'Schema shipments'!$B$10</definedName>
+    <definedName name="schema.physicalType" localSheetId="2">'Schema shipments'!$B$6</definedName>
+    <definedName name="schema.properties" localSheetId="2">'Schema shipments'!$A$17:$AW$985</definedName>
+    <definedName name="schema.tags" localSheetId="2">'Schema shipments'!$B$12</definedName>
     <definedName name="servers.account">Servers!$C$11</definedName>
     <definedName name="servers.catalog">Servers!$C$12</definedName>
     <definedName name="servers.catalogUrl">Servers!$C$13</definedName>
@@ -133,7 +133,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="812" uniqueCount="437">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="811" uniqueCount="437">
   <si>
     <t>Fundamentals</t>
   </si>
@@ -1669,7 +1669,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1757,8 +1757,10 @@
     <xf numFmtId="49" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -1773,10 +1775,6 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -16168,10 +16166,10 @@
       <c r="B12" s="7"/>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A13" s="43" t="s">
+      <c r="A13" s="35" t="s">
         <v>15</v>
       </c>
-      <c r="B13" s="44"/>
+      <c r="B13" s="36"/>
       <c r="C13" s="5" t="s">
         <v>16</v>
       </c>
@@ -16292,7 +16290,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:AZ54"/>
+  <dimension ref="A1:AZ53"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="34.83203125" style="2" customWidth="1"/>
@@ -16320,22 +16318,22 @@
     <col min="54" max="16384" width="8.83203125" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:52" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A3" s="4" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A5" s="7" t="s">
         <v>8</v>
       </c>
@@ -16346,327 +16344,406 @@
       <c r="D5" s="38"/>
       <c r="E5" s="39"/>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A6" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="B6" s="5"/>
-      <c r="C6" s="35"/>
-      <c r="D6" s="35"/>
-      <c r="E6" s="36"/>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+        <v>61</v>
+      </c>
+      <c r="B6" s="37" t="s">
+        <v>62</v>
+      </c>
+      <c r="C6" s="38"/>
+      <c r="D6" s="38"/>
+      <c r="E6" s="39"/>
+    </row>
+    <row r="7" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A7" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="B7" s="37" t="s">
-        <v>62</v>
-      </c>
-      <c r="C7" s="38"/>
-      <c r="D7" s="38"/>
-      <c r="E7" s="39"/>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+        <v>76</v>
+      </c>
+      <c r="B7" s="40"/>
+      <c r="C7" s="41"/>
+      <c r="D7" s="41"/>
+      <c r="E7" s="42"/>
+    </row>
+    <row r="8" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A8" s="7" t="s">
-        <v>76</v>
-      </c>
-      <c r="B8" s="40"/>
-      <c r="C8" s="41"/>
-      <c r="D8" s="41"/>
-      <c r="E8" s="42"/>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+        <v>22</v>
+      </c>
+      <c r="B8" s="37" t="s">
+        <v>63</v>
+      </c>
+      <c r="C8" s="38"/>
+      <c r="D8" s="38"/>
+      <c r="E8" s="39"/>
+    </row>
+    <row r="9" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A9" s="7" t="s">
-        <v>22</v>
+        <v>64</v>
       </c>
       <c r="B9" s="37" t="s">
-        <v>63</v>
+        <v>9</v>
       </c>
       <c r="C9" s="38"/>
       <c r="D9" s="38"/>
       <c r="E9" s="39"/>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A10" s="7" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B10" s="37" t="s">
-        <v>9</v>
+        <v>66</v>
       </c>
       <c r="C10" s="38"/>
       <c r="D10" s="38"/>
       <c r="E10" s="39"/>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A11" s="7" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B11" s="37" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C11" s="38"/>
       <c r="D11" s="38"/>
       <c r="E11" s="39"/>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A12" s="7" t="s">
-        <v>67</v>
+        <v>29</v>
       </c>
       <c r="B12" s="37" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C12" s="38"/>
       <c r="D12" s="38"/>
       <c r="E12" s="39"/>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A13" s="7" t="s">
-        <v>29</v>
+        <v>6</v>
       </c>
       <c r="B13" s="37" t="s">
-        <v>69</v>
+        <v>60</v>
       </c>
       <c r="C13" s="38"/>
       <c r="D13" s="38"/>
       <c r="E13" s="39"/>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A14" s="7" t="s">
-        <v>6</v>
+        <v>70</v>
       </c>
       <c r="B14" s="37" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="C14" s="38"/>
       <c r="D14" s="38"/>
       <c r="E14" s="39"/>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A15" s="7" t="s">
-        <v>70</v>
-      </c>
-      <c r="B15" s="37" t="s">
-        <v>71</v>
-      </c>
+        <v>72</v>
+      </c>
+      <c r="B15" s="37"/>
       <c r="C15" s="38"/>
       <c r="D15" s="38"/>
       <c r="E15" s="39"/>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A16" s="7" t="s">
+    <row r="16" spans="1:52" x14ac:dyDescent="0.2">
+      <c r="E16" s="2"/>
+      <c r="Y16" s="19" t="s">
+        <v>73</v>
+      </c>
+      <c r="Z16" s="20"/>
+      <c r="AA16" s="20"/>
+      <c r="AB16" s="20"/>
+      <c r="AC16" s="20"/>
+      <c r="AD16" s="20"/>
+      <c r="AE16" s="20"/>
+      <c r="AF16" s="20"/>
+      <c r="AG16" s="20"/>
+      <c r="AH16" s="20"/>
+      <c r="AI16" s="20"/>
+      <c r="AJ16" s="20"/>
+      <c r="AK16" s="20"/>
+      <c r="AL16" s="20"/>
+      <c r="AM16" s="20"/>
+      <c r="AN16" s="20"/>
+      <c r="AO16" s="20"/>
+      <c r="AP16" s="20"/>
+      <c r="AQ16" s="20"/>
+      <c r="AR16" s="20"/>
+      <c r="AS16" s="20"/>
+      <c r="AT16" s="20"/>
+      <c r="AU16" s="21"/>
+      <c r="AX16" s="19" t="s">
+        <v>74</v>
+      </c>
+      <c r="AY16" s="20"/>
+      <c r="AZ16" s="20"/>
+    </row>
+    <row r="17" spans="1:52" x14ac:dyDescent="0.2">
+      <c r="A17" s="9" t="s">
+        <v>75</v>
+      </c>
+      <c r="B17" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="C17" s="10" t="s">
+        <v>76</v>
+      </c>
+      <c r="D17" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="E17" s="11" t="s">
+        <v>78</v>
+      </c>
+      <c r="F17" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="G17" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="H17" s="10" t="s">
+        <v>80</v>
+      </c>
+      <c r="I17" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="J17" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="K17" s="10" t="s">
+        <v>82</v>
+      </c>
+      <c r="L17" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="B16" s="37"/>
-      <c r="C16" s="38"/>
-      <c r="D16" s="38"/>
-      <c r="E16" s="39"/>
-    </row>
-    <row r="17" spans="1:52" x14ac:dyDescent="0.2">
-      <c r="E17" s="2"/>
-      <c r="Y17" s="19" t="s">
-        <v>73</v>
-      </c>
-      <c r="Z17" s="20"/>
-      <c r="AA17" s="20"/>
-      <c r="AB17" s="20"/>
-      <c r="AC17" s="20"/>
-      <c r="AD17" s="20"/>
-      <c r="AE17" s="20"/>
-      <c r="AF17" s="20"/>
-      <c r="AG17" s="20"/>
-      <c r="AH17" s="20"/>
-      <c r="AI17" s="20"/>
-      <c r="AJ17" s="20"/>
-      <c r="AK17" s="20"/>
-      <c r="AL17" s="20"/>
-      <c r="AM17" s="20"/>
-      <c r="AN17" s="20"/>
-      <c r="AO17" s="20"/>
-      <c r="AP17" s="20"/>
-      <c r="AQ17" s="20"/>
-      <c r="AR17" s="20"/>
-      <c r="AS17" s="20"/>
-      <c r="AT17" s="20"/>
-      <c r="AU17" s="21"/>
-      <c r="AX17" s="19" t="s">
-        <v>74</v>
-      </c>
-      <c r="AY17" s="20"/>
-      <c r="AZ17" s="20"/>
-    </row>
-    <row r="18" spans="1:52" x14ac:dyDescent="0.2">
-      <c r="A18" s="9" t="s">
-        <v>75</v>
-      </c>
-      <c r="B18" s="10" t="s">
-        <v>64</v>
-      </c>
-      <c r="C18" s="10" t="s">
-        <v>76</v>
-      </c>
-      <c r="D18" s="10" t="s">
-        <v>77</v>
-      </c>
-      <c r="E18" s="11" t="s">
-        <v>78</v>
-      </c>
-      <c r="F18" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="G18" s="10" t="s">
-        <v>79</v>
-      </c>
-      <c r="H18" s="10" t="s">
-        <v>80</v>
-      </c>
-      <c r="I18" s="10" t="s">
-        <v>81</v>
-      </c>
-      <c r="J18" s="10" t="s">
-        <v>29</v>
-      </c>
-      <c r="K18" s="10" t="s">
-        <v>82</v>
-      </c>
-      <c r="L18" s="10" t="s">
-        <v>72</v>
-      </c>
-      <c r="M18" s="10" t="s">
+      <c r="M17" s="10" t="s">
         <v>83</v>
       </c>
-      <c r="N18" s="10" t="s">
+      <c r="N17" s="10" t="s">
         <v>84</v>
       </c>
-      <c r="O18" s="10" t="s">
+      <c r="O17" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="P18" s="10" t="s">
+      <c r="P17" s="10" t="s">
         <v>85</v>
       </c>
-      <c r="Q18" s="10" t="s">
+      <c r="Q17" s="10" t="s">
         <v>86</v>
       </c>
-      <c r="R18" s="10" t="s">
+      <c r="R17" s="10" t="s">
         <v>87</v>
       </c>
-      <c r="S18" s="10" t="s">
+      <c r="S17" s="10" t="s">
         <v>88</v>
       </c>
-      <c r="T18" s="10" t="s">
+      <c r="T17" s="10" t="s">
         <v>89</v>
       </c>
-      <c r="U18" s="10" t="s">
+      <c r="U17" s="10" t="s">
         <v>90</v>
       </c>
-      <c r="V18" s="10" t="s">
+      <c r="V17" s="10" t="s">
         <v>91</v>
       </c>
-      <c r="W18" s="10" t="s">
+      <c r="W17" s="10" t="s">
         <v>92</v>
       </c>
-      <c r="X18" s="10" t="s">
+      <c r="X17" s="10" t="s">
         <v>93</v>
       </c>
-      <c r="Y18" s="10" t="s">
+      <c r="Y17" s="10" t="s">
         <v>94</v>
       </c>
-      <c r="Z18" s="10" t="s">
+      <c r="Z17" s="10" t="s">
         <v>95</v>
       </c>
-      <c r="AA18" s="10" t="s">
+      <c r="AA17" s="10" t="s">
         <v>96</v>
       </c>
-      <c r="AB18" s="10" t="s">
+      <c r="AB17" s="10" t="s">
         <v>97</v>
       </c>
-      <c r="AC18" s="10" t="s">
+      <c r="AC17" s="10" t="s">
         <v>98</v>
       </c>
-      <c r="AD18" s="10" t="s">
+      <c r="AD17" s="10" t="s">
         <v>99</v>
       </c>
-      <c r="AE18" s="10" t="s">
+      <c r="AE17" s="10" t="s">
         <v>100</v>
       </c>
-      <c r="AF18" s="10" t="s">
+      <c r="AF17" s="10" t="s">
         <v>101</v>
       </c>
-      <c r="AG18" s="10" t="s">
+      <c r="AG17" s="10" t="s">
         <v>102</v>
       </c>
-      <c r="AH18" s="10" t="s">
+      <c r="AH17" s="10" t="s">
         <v>103</v>
       </c>
-      <c r="AI18" s="10" t="s">
+      <c r="AI17" s="10" t="s">
         <v>104</v>
       </c>
-      <c r="AJ18" s="10" t="s">
+      <c r="AJ17" s="10" t="s">
         <v>105</v>
       </c>
-      <c r="AK18" s="10" t="s">
+      <c r="AK17" s="10" t="s">
         <v>106</v>
       </c>
-      <c r="AL18" s="10" t="s">
+      <c r="AL17" s="10" t="s">
         <v>107</v>
       </c>
-      <c r="AM18" s="10" t="s">
+      <c r="AM17" s="10" t="s">
         <v>108</v>
       </c>
-      <c r="AN18" s="10" t="s">
+      <c r="AN17" s="10" t="s">
         <v>109</v>
       </c>
-      <c r="AO18" s="10" t="s">
+      <c r="AO17" s="10" t="s">
         <v>110</v>
       </c>
-      <c r="AP18" s="10" t="s">
+      <c r="AP17" s="10" t="s">
         <v>111</v>
       </c>
-      <c r="AQ18" s="10" t="s">
+      <c r="AQ17" s="10" t="s">
         <v>112</v>
       </c>
-      <c r="AR18" s="10" t="s">
+      <c r="AR17" s="10" t="s">
         <v>113</v>
       </c>
-      <c r="AS18" s="10" t="s">
+      <c r="AS17" s="10" t="s">
         <v>114</v>
       </c>
-      <c r="AT18" s="10" t="s">
+      <c r="AT17" s="10" t="s">
         <v>115</v>
       </c>
-      <c r="AU18" s="10" t="s">
+      <c r="AU17" s="10" t="s">
         <v>116</v>
       </c>
-      <c r="AV18" s="10" t="s">
+      <c r="AV17" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="AW18" s="10" t="s">
+      <c r="AW17" s="10" t="s">
         <v>117</v>
       </c>
-      <c r="AX18" s="10"/>
-      <c r="AY18" s="10"/>
-      <c r="AZ18" s="10"/>
+      <c r="AX17" s="10"/>
+      <c r="AY17" s="10"/>
+      <c r="AZ17" s="10"/>
+    </row>
+    <row r="18" spans="1:52" ht="34" x14ac:dyDescent="0.2">
+      <c r="A18" s="17" t="s">
+        <v>118</v>
+      </c>
+      <c r="B18" s="15" t="s">
+        <v>119</v>
+      </c>
+      <c r="C18" s="15" t="s">
+        <v>120</v>
+      </c>
+      <c r="D18" s="15" t="s">
+        <v>121</v>
+      </c>
+      <c r="E18" s="16" t="s">
+        <v>122</v>
+      </c>
+      <c r="F18" s="15" t="s">
+        <v>123</v>
+      </c>
+      <c r="G18" s="15" t="b">
+        <v>0</v>
+      </c>
+      <c r="H18" s="15" t="b">
+        <v>0</v>
+      </c>
+      <c r="I18" s="15" t="s">
+        <v>124</v>
+      </c>
+      <c r="J18" s="15" t="s">
+        <v>125</v>
+      </c>
+      <c r="K18" s="15"/>
+      <c r="L18" s="15"/>
+      <c r="M18" s="15" t="s">
+        <v>126</v>
+      </c>
+      <c r="N18" s="15" t="s">
+        <v>127</v>
+      </c>
+      <c r="O18" s="15" t="s">
+        <v>128</v>
+      </c>
+      <c r="P18" s="15" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q18" s="15"/>
+      <c r="R18" s="15" t="b">
+        <v>0</v>
+      </c>
+      <c r="S18" s="15"/>
+      <c r="T18" s="15"/>
+      <c r="U18" s="15"/>
+      <c r="V18" s="15"/>
+      <c r="W18" s="15"/>
+      <c r="X18" s="15" t="b">
+        <v>0</v>
+      </c>
+      <c r="Y18" s="15"/>
+      <c r="Z18" s="15"/>
+      <c r="AA18" s="15"/>
+      <c r="AB18" s="15"/>
+      <c r="AC18" s="15"/>
+      <c r="AD18" s="15"/>
+      <c r="AE18" s="16"/>
+      <c r="AF18" s="16"/>
+      <c r="AG18" s="16"/>
+      <c r="AH18" s="16"/>
+      <c r="AI18" s="15"/>
+      <c r="AJ18" s="15"/>
+      <c r="AK18" s="15"/>
+      <c r="AL18" s="15"/>
+      <c r="AM18" s="15"/>
+      <c r="AN18" s="15"/>
+      <c r="AO18" s="15"/>
+      <c r="AP18" s="15"/>
+      <c r="AQ18" s="15"/>
+      <c r="AR18" s="15"/>
+      <c r="AS18" s="15"/>
+      <c r="AT18" s="15"/>
+      <c r="AU18" s="15"/>
+      <c r="AV18" s="15" t="s">
+        <v>118</v>
+      </c>
+      <c r="AW18" s="28"/>
+      <c r="AX18" s="15"/>
+      <c r="AY18" s="15"/>
+      <c r="AZ18" s="15"/>
     </row>
     <row r="19" spans="1:52" ht="34" x14ac:dyDescent="0.2">
       <c r="A19" s="17" t="s">
-        <v>118</v>
+        <v>129</v>
       </c>
       <c r="B19" s="15" t="s">
-        <v>119</v>
+        <v>130</v>
       </c>
       <c r="C19" s="15" t="s">
         <v>120</v>
       </c>
       <c r="D19" s="15" t="s">
-        <v>121</v>
+        <v>131</v>
       </c>
       <c r="E19" s="16" t="s">
-        <v>122</v>
+        <v>132</v>
       </c>
       <c r="F19" s="15" t="s">
-        <v>123</v>
+        <v>133</v>
       </c>
       <c r="G19" s="15" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H19" s="15" t="b">
         <v>0</v>
@@ -16674,22 +16751,16 @@
       <c r="I19" s="15" t="s">
         <v>124</v>
       </c>
-      <c r="J19" s="15" t="s">
-        <v>125</v>
-      </c>
+      <c r="J19" s="15"/>
       <c r="K19" s="15"/>
       <c r="L19" s="15"/>
-      <c r="M19" s="15" t="s">
-        <v>126</v>
-      </c>
-      <c r="N19" s="15" t="s">
-        <v>127</v>
-      </c>
+      <c r="M19" s="15"/>
+      <c r="N19" s="15"/>
       <c r="O19" s="15" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="P19" s="15" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q19" s="15"/>
       <c r="R19" s="15" t="b">
@@ -16707,8 +16778,12 @@
       <c r="Z19" s="15"/>
       <c r="AA19" s="15"/>
       <c r="AB19" s="15"/>
-      <c r="AC19" s="15"/>
-      <c r="AD19" s="15"/>
+      <c r="AC19" s="15">
+        <v>8</v>
+      </c>
+      <c r="AD19" s="15">
+        <v>10</v>
+      </c>
       <c r="AE19" s="16"/>
       <c r="AF19" s="16"/>
       <c r="AG19" s="16"/>
@@ -16727,7 +16802,7 @@
       <c r="AT19" s="15"/>
       <c r="AU19" s="15"/>
       <c r="AV19" s="15" t="s">
-        <v>118</v>
+        <v>129</v>
       </c>
       <c r="AW19" s="28"/>
       <c r="AX19" s="15"/>
@@ -16736,25 +16811,25 @@
     </row>
     <row r="20" spans="1:52" ht="34" x14ac:dyDescent="0.2">
       <c r="A20" s="17" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="B20" s="15" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="C20" s="15" t="s">
-        <v>120</v>
+        <v>137</v>
       </c>
       <c r="D20" s="15" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="E20" s="16" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
       <c r="F20" s="15" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="G20" s="15" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H20" s="15" t="b">
         <v>0</v>
@@ -16767,9 +16842,7 @@
       <c r="L20" s="15"/>
       <c r="M20" s="15"/>
       <c r="N20" s="15"/>
-      <c r="O20" s="15" t="s">
-        <v>134</v>
-      </c>
+      <c r="O20" s="15"/>
       <c r="P20" s="15" t="b">
         <v>0</v>
       </c>
@@ -16789,12 +16862,8 @@
       <c r="Z20" s="15"/>
       <c r="AA20" s="15"/>
       <c r="AB20" s="15"/>
-      <c r="AC20" s="15">
-        <v>8</v>
-      </c>
-      <c r="AD20" s="15">
-        <v>10</v>
-      </c>
+      <c r="AC20" s="15"/>
+      <c r="AD20" s="15"/>
       <c r="AE20" s="16"/>
       <c r="AF20" s="16"/>
       <c r="AG20" s="16"/>
@@ -16812,9 +16881,7 @@
       <c r="AS20" s="15"/>
       <c r="AT20" s="15"/>
       <c r="AU20" s="15"/>
-      <c r="AV20" s="15" t="s">
-        <v>129</v>
-      </c>
+      <c r="AV20" s="15"/>
       <c r="AW20" s="28"/>
       <c r="AX20" s="15"/>
       <c r="AY20" s="15"/>
@@ -16822,22 +16889,22 @@
     </row>
     <row r="21" spans="1:52" ht="34" x14ac:dyDescent="0.2">
       <c r="A21" s="17" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="B21" s="15" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="C21" s="15" t="s">
-        <v>137</v>
+        <v>120</v>
       </c>
       <c r="D21" s="15" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="E21" s="16" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="F21" s="15" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="G21" s="15" t="b">
         <v>0</v>
@@ -16849,7 +16916,9 @@
         <v>124</v>
       </c>
       <c r="J21" s="15"/>
-      <c r="K21" s="15"/>
+      <c r="K21" s="15" t="s">
+        <v>145</v>
+      </c>
       <c r="L21" s="15"/>
       <c r="M21" s="15"/>
       <c r="N21" s="15"/>
@@ -16900,10 +16969,10 @@
     </row>
     <row r="22" spans="1:52" ht="34" x14ac:dyDescent="0.2">
       <c r="A22" s="17" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="B22" s="15" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="C22" s="15" t="s">
         <v>120</v>
@@ -16912,10 +16981,10 @@
         <v>131</v>
       </c>
       <c r="E22" s="16" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="F22" s="15" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="G22" s="15" t="b">
         <v>0</v>
@@ -16924,12 +16993,10 @@
         <v>0</v>
       </c>
       <c r="I22" s="15" t="s">
-        <v>124</v>
+        <v>150</v>
       </c>
       <c r="J22" s="15"/>
-      <c r="K22" s="15" t="s">
-        <v>145</v>
-      </c>
+      <c r="K22" s="15"/>
       <c r="L22" s="15"/>
       <c r="M22" s="15"/>
       <c r="N22" s="15"/>
@@ -16978,12 +17045,12 @@
       <c r="AY22" s="15"/>
       <c r="AZ22" s="15"/>
     </row>
-    <row r="23" spans="1:52" ht="34" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:52" ht="17" x14ac:dyDescent="0.2">
       <c r="A23" s="17" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="B23" s="15" t="s">
-        <v>147</v>
+        <v>12</v>
       </c>
       <c r="C23" s="15" t="s">
         <v>120</v>
@@ -16992,10 +17059,10 @@
         <v>131</v>
       </c>
       <c r="E23" s="16" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="F23" s="15" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="G23" s="15" t="b">
         <v>0</v>
@@ -17004,10 +17071,12 @@
         <v>0</v>
       </c>
       <c r="I23" s="15" t="s">
-        <v>150</v>
+        <v>124</v>
       </c>
       <c r="J23" s="15"/>
-      <c r="K23" s="15"/>
+      <c r="K23" s="15" t="s">
+        <v>145</v>
+      </c>
       <c r="L23" s="15"/>
       <c r="M23" s="15"/>
       <c r="N23" s="15"/>
@@ -17056,12 +17125,12 @@
       <c r="AY23" s="15"/>
       <c r="AZ23" s="15"/>
     </row>
-    <row r="24" spans="1:52" ht="17" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:52" ht="34" x14ac:dyDescent="0.2">
       <c r="A24" s="17" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="B24" s="15" t="s">
-        <v>12</v>
+        <v>155</v>
       </c>
       <c r="C24" s="15" t="s">
         <v>120</v>
@@ -17070,43 +17139,35 @@
         <v>131</v>
       </c>
       <c r="E24" s="16" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="F24" s="15" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="G24" s="15" t="b">
         <v>0</v>
       </c>
-      <c r="H24" s="15" t="b">
-        <v>0</v>
-      </c>
+      <c r="H24" s="15"/>
       <c r="I24" s="15" t="s">
         <v>124</v>
       </c>
       <c r="J24" s="15"/>
-      <c r="K24" s="15" t="s">
-        <v>145</v>
-      </c>
-      <c r="L24" s="15"/>
+      <c r="K24" s="15"/>
+      <c r="L24" s="15" t="b">
+        <v>1</v>
+      </c>
       <c r="M24" s="15"/>
       <c r="N24" s="15"/>
       <c r="O24" s="15"/>
-      <c r="P24" s="15" t="b">
-        <v>0</v>
-      </c>
+      <c r="P24" s="15"/>
       <c r="Q24" s="15"/>
-      <c r="R24" s="15" t="b">
-        <v>0</v>
-      </c>
+      <c r="R24" s="15"/>
       <c r="S24" s="15"/>
       <c r="T24" s="15"/>
       <c r="U24" s="15"/>
       <c r="V24" s="15"/>
       <c r="W24" s="15"/>
-      <c r="X24" s="15" t="b">
-        <v>0</v>
-      </c>
+      <c r="X24" s="15"/>
       <c r="Y24" s="15"/>
       <c r="Z24" s="15"/>
       <c r="AA24" s="15"/>
@@ -17136,24 +17197,24 @@
       <c r="AY24" s="15"/>
       <c r="AZ24" s="15"/>
     </row>
-    <row r="25" spans="1:52" ht="34" x14ac:dyDescent="0.2">
-      <c r="A25" s="17" t="s">
-        <v>154</v>
+    <row r="25" spans="1:52" ht="51" x14ac:dyDescent="0.2">
+      <c r="A25" s="18" t="s">
+        <v>158</v>
       </c>
       <c r="B25" s="15" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="C25" s="15" t="s">
-        <v>120</v>
+        <v>160</v>
       </c>
       <c r="D25" s="15" t="s">
-        <v>131</v>
-      </c>
-      <c r="E25" s="16" t="s">
-        <v>156</v>
+        <v>161</v>
+      </c>
+      <c r="E25" s="16">
+        <v>12.5</v>
       </c>
       <c r="F25" s="15" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
       <c r="G25" s="15" t="b">
         <v>0</v>
@@ -17163,10 +17224,10 @@
         <v>124</v>
       </c>
       <c r="J25" s="15"/>
-      <c r="K25" s="15"/>
-      <c r="L25" s="15" t="b">
-        <v>1</v>
-      </c>
+      <c r="K25" s="15" t="s">
+        <v>163</v>
+      </c>
+      <c r="L25" s="15"/>
       <c r="M25" s="15"/>
       <c r="N25" s="15"/>
       <c r="O25" s="15"/>
@@ -17176,8 +17237,12 @@
       <c r="S25" s="15"/>
       <c r="T25" s="15"/>
       <c r="U25" s="15"/>
-      <c r="V25" s="15"/>
-      <c r="W25" s="15"/>
+      <c r="V25" s="15" t="s">
+        <v>164</v>
+      </c>
+      <c r="W25" s="15" t="s">
+        <v>165</v>
+      </c>
       <c r="X25" s="15"/>
       <c r="Y25" s="15"/>
       <c r="Z25" s="15"/>
@@ -17208,53 +17273,57 @@
       <c r="AY25" s="15"/>
       <c r="AZ25" s="15"/>
     </row>
-    <row r="26" spans="1:52" ht="51" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:52" ht="34" x14ac:dyDescent="0.2">
       <c r="A26" s="18" t="s">
-        <v>158</v>
+        <v>166</v>
       </c>
       <c r="B26" s="15" t="s">
-        <v>159</v>
+        <v>167</v>
       </c>
       <c r="C26" s="15" t="s">
-        <v>160</v>
+        <v>168</v>
       </c>
       <c r="D26" s="15" t="s">
-        <v>161</v>
-      </c>
-      <c r="E26" s="16">
-        <v>12.5</v>
+        <v>169</v>
+      </c>
+      <c r="E26" s="16" t="s">
+        <v>170</v>
       </c>
       <c r="F26" s="15" t="s">
-        <v>162</v>
+        <v>171</v>
       </c>
       <c r="G26" s="15" t="b">
         <v>0</v>
       </c>
-      <c r="H26" s="15"/>
+      <c r="H26" s="15" t="b">
+        <v>0</v>
+      </c>
       <c r="I26" s="15" t="s">
         <v>124</v>
       </c>
       <c r="J26" s="15"/>
-      <c r="K26" s="15" t="s">
-        <v>163</v>
-      </c>
+      <c r="K26" s="15"/>
       <c r="L26" s="15"/>
       <c r="M26" s="15"/>
       <c r="N26" s="15"/>
       <c r="O26" s="15"/>
-      <c r="P26" s="15"/>
+      <c r="P26" s="15" t="b">
+        <v>0</v>
+      </c>
       <c r="Q26" s="15"/>
-      <c r="R26" s="15"/>
-      <c r="S26" s="15"/>
+      <c r="R26" s="15" t="b">
+        <v>0</v>
+      </c>
+      <c r="S26" s="15">
+        <v>-1</v>
+      </c>
       <c r="T26" s="15"/>
       <c r="U26" s="15"/>
-      <c r="V26" s="15" t="s">
-        <v>164</v>
-      </c>
-      <c r="W26" s="15" t="s">
-        <v>165</v>
-      </c>
-      <c r="X26" s="15"/>
+      <c r="V26" s="15"/>
+      <c r="W26" s="15"/>
+      <c r="X26" s="15" t="b">
+        <v>0</v>
+      </c>
       <c r="Y26" s="15"/>
       <c r="Z26" s="15"/>
       <c r="AA26" s="15"/>
@@ -17284,33 +17353,29 @@
       <c r="AY26" s="15"/>
       <c r="AZ26" s="15"/>
     </row>
-    <row r="27" spans="1:52" ht="34" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:52" ht="17" x14ac:dyDescent="0.2">
       <c r="A27" s="18" t="s">
-        <v>166</v>
+        <v>172</v>
       </c>
       <c r="B27" s="15" t="s">
-        <v>167</v>
+        <v>173</v>
       </c>
       <c r="C27" s="15" t="s">
         <v>168</v>
       </c>
       <c r="D27" s="15" t="s">
-        <v>169</v>
-      </c>
-      <c r="E27" s="16" t="s">
-        <v>170</v>
-      </c>
+        <v>174</v>
+      </c>
+      <c r="E27" s="16"/>
       <c r="F27" s="15" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="G27" s="15" t="b">
-        <v>0</v>
-      </c>
-      <c r="H27" s="15" t="b">
-        <v>0</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="H27" s="15"/>
       <c r="I27" s="15" t="s">
-        <v>124</v>
+        <v>150</v>
       </c>
       <c r="J27" s="15"/>
       <c r="K27" s="15"/>
@@ -17318,23 +17383,15 @@
       <c r="M27" s="15"/>
       <c r="N27" s="15"/>
       <c r="O27" s="15"/>
-      <c r="P27" s="15" t="b">
-        <v>0</v>
-      </c>
+      <c r="P27" s="15"/>
       <c r="Q27" s="15"/>
-      <c r="R27" s="15" t="b">
-        <v>0</v>
-      </c>
-      <c r="S27" s="15">
-        <v>-1</v>
-      </c>
+      <c r="R27" s="15"/>
+      <c r="S27" s="15"/>
       <c r="T27" s="15"/>
       <c r="U27" s="15"/>
       <c r="V27" s="15"/>
       <c r="W27" s="15"/>
-      <c r="X27" s="15" t="b">
-        <v>0</v>
-      </c>
+      <c r="X27" s="15"/>
       <c r="Y27" s="15"/>
       <c r="Z27" s="15"/>
       <c r="AA27" s="15"/>
@@ -17365,26 +17422,30 @@
       <c r="AZ27" s="15"/>
     </row>
     <row r="28" spans="1:52" ht="17" x14ac:dyDescent="0.2">
-      <c r="A28" s="18" t="s">
-        <v>172</v>
+      <c r="A28" s="17" t="s">
+        <v>176</v>
       </c>
       <c r="B28" s="15" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="C28" s="15" t="s">
-        <v>168</v>
+        <v>120</v>
       </c>
       <c r="D28" s="15" t="s">
-        <v>174</v>
-      </c>
-      <c r="E28" s="16"/>
+        <v>131</v>
+      </c>
+      <c r="E28" s="16" t="s">
+        <v>178</v>
+      </c>
       <c r="F28" s="15" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="G28" s="15" t="b">
         <v>1</v>
       </c>
-      <c r="H28" s="15"/>
+      <c r="H28" s="15" t="b">
+        <v>0</v>
+      </c>
       <c r="I28" s="15" t="s">
         <v>150</v>
       </c>
@@ -17394,9 +17455,13 @@
       <c r="M28" s="15"/>
       <c r="N28" s="15"/>
       <c r="O28" s="15"/>
-      <c r="P28" s="15"/>
+      <c r="P28" s="15" t="b">
+        <v>0</v>
+      </c>
       <c r="Q28" s="15"/>
-      <c r="R28" s="15"/>
+      <c r="R28" s="15" t="b">
+        <v>0</v>
+      </c>
       <c r="S28" s="15"/>
       <c r="T28" s="15"/>
       <c r="U28" s="15"/>
@@ -17434,10 +17499,10 @@
     </row>
     <row r="29" spans="1:52" ht="17" x14ac:dyDescent="0.2">
       <c r="A29" s="17" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="B29" s="15" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="C29" s="15" t="s">
         <v>120</v>
@@ -17446,10 +17511,10 @@
         <v>131</v>
       </c>
       <c r="E29" s="16" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="F29" s="15" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="G29" s="15" t="b">
         <v>1</v>
@@ -17510,10 +17575,10 @@
     </row>
     <row r="30" spans="1:52" ht="17" x14ac:dyDescent="0.2">
       <c r="A30" s="17" t="s">
-        <v>180</v>
+        <v>184</v>
       </c>
       <c r="B30" s="15" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="C30" s="15" t="s">
         <v>120</v>
@@ -17522,22 +17587,22 @@
         <v>131</v>
       </c>
       <c r="E30" s="16" t="s">
-        <v>182</v>
+        <v>186</v>
       </c>
       <c r="F30" s="15" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
       <c r="G30" s="15" t="b">
         <v>1</v>
       </c>
-      <c r="H30" s="15" t="b">
-        <v>0</v>
-      </c>
+      <c r="H30" s="15"/>
       <c r="I30" s="15" t="s">
         <v>150</v>
       </c>
       <c r="J30" s="15"/>
-      <c r="K30" s="15"/>
+      <c r="K30" s="15" t="s">
+        <v>145</v>
+      </c>
       <c r="L30" s="15"/>
       <c r="M30" s="15"/>
       <c r="N30" s="15"/>
@@ -17584,47 +17649,25 @@
       <c r="AY30" s="15"/>
       <c r="AZ30" s="15"/>
     </row>
-    <row r="31" spans="1:52" ht="17" x14ac:dyDescent="0.2">
-      <c r="A31" s="17" t="s">
-        <v>184</v>
-      </c>
-      <c r="B31" s="15" t="s">
-        <v>185</v>
-      </c>
-      <c r="C31" s="15" t="s">
-        <v>120</v>
-      </c>
-      <c r="D31" s="15" t="s">
-        <v>131</v>
-      </c>
-      <c r="E31" s="16" t="s">
-        <v>186</v>
-      </c>
-      <c r="F31" s="15" t="s">
-        <v>187</v>
-      </c>
-      <c r="G31" s="15" t="b">
-        <v>1</v>
-      </c>
+    <row r="31" spans="1:52" x14ac:dyDescent="0.2">
+      <c r="A31" s="17"/>
+      <c r="B31" s="15"/>
+      <c r="C31" s="15"/>
+      <c r="D31" s="15"/>
+      <c r="E31" s="16"/>
+      <c r="F31" s="15"/>
+      <c r="G31" s="15"/>
       <c r="H31" s="15"/>
-      <c r="I31" s="15" t="s">
-        <v>150</v>
-      </c>
+      <c r="I31" s="15"/>
       <c r="J31" s="15"/>
-      <c r="K31" s="15" t="s">
-        <v>145</v>
-      </c>
+      <c r="K31" s="15"/>
       <c r="L31" s="15"/>
       <c r="M31" s="15"/>
       <c r="N31" s="15"/>
       <c r="O31" s="15"/>
-      <c r="P31" s="15" t="b">
-        <v>0</v>
-      </c>
+      <c r="P31" s="15"/>
       <c r="Q31" s="15"/>
-      <c r="R31" s="15" t="b">
-        <v>0</v>
-      </c>
+      <c r="R31" s="15"/>
       <c r="S31" s="15"/>
       <c r="T31" s="15"/>
       <c r="U31" s="15"/>
@@ -18848,117 +18891,63 @@
       <c r="AY53" s="15"/>
       <c r="AZ53" s="15"/>
     </row>
-    <row r="54" spans="1:52" x14ac:dyDescent="0.2">
-      <c r="A54" s="17"/>
-      <c r="B54" s="15"/>
-      <c r="C54" s="15"/>
-      <c r="D54" s="15"/>
-      <c r="E54" s="16"/>
-      <c r="F54" s="15"/>
-      <c r="G54" s="15"/>
-      <c r="H54" s="15"/>
-      <c r="I54" s="15"/>
-      <c r="J54" s="15"/>
-      <c r="K54" s="15"/>
-      <c r="L54" s="15"/>
-      <c r="M54" s="15"/>
-      <c r="N54" s="15"/>
-      <c r="O54" s="15"/>
-      <c r="P54" s="15"/>
-      <c r="Q54" s="15"/>
-      <c r="R54" s="15"/>
-      <c r="S54" s="15"/>
-      <c r="T54" s="15"/>
-      <c r="U54" s="15"/>
-      <c r="V54" s="15"/>
-      <c r="W54" s="15"/>
-      <c r="X54" s="15"/>
-      <c r="Y54" s="15"/>
-      <c r="Z54" s="15"/>
-      <c r="AA54" s="15"/>
-      <c r="AB54" s="15"/>
-      <c r="AC54" s="15"/>
-      <c r="AD54" s="15"/>
-      <c r="AE54" s="16"/>
-      <c r="AF54" s="16"/>
-      <c r="AG54" s="16"/>
-      <c r="AH54" s="16"/>
-      <c r="AI54" s="15"/>
-      <c r="AJ54" s="15"/>
-      <c r="AK54" s="15"/>
-      <c r="AL54" s="15"/>
-      <c r="AM54" s="15"/>
-      <c r="AN54" s="15"/>
-      <c r="AO54" s="15"/>
-      <c r="AP54" s="15"/>
-      <c r="AQ54" s="15"/>
-      <c r="AR54" s="15"/>
-      <c r="AS54" s="15"/>
-      <c r="AT54" s="15"/>
-      <c r="AU54" s="15"/>
-      <c r="AV54" s="15"/>
-      <c r="AW54" s="28"/>
-      <c r="AX54" s="15"/>
-      <c r="AY54" s="15"/>
-      <c r="AZ54" s="15"/>
-    </row>
   </sheetData>
   <mergeCells count="11">
     <mergeCell ref="B5:E5"/>
-    <mergeCell ref="B12:E12"/>
-    <mergeCell ref="B16:E16"/>
-    <mergeCell ref="B8:E8"/>
     <mergeCell ref="B11:E11"/>
-    <mergeCell ref="B10:E10"/>
-    <mergeCell ref="B14:E14"/>
     <mergeCell ref="B15:E15"/>
     <mergeCell ref="B7:E7"/>
+    <mergeCell ref="B10:E10"/>
     <mergeCell ref="B9:E9"/>
     <mergeCell ref="B13:E13"/>
+    <mergeCell ref="B14:E14"/>
+    <mergeCell ref="B6:E6"/>
+    <mergeCell ref="B8:E8"/>
+    <mergeCell ref="B12:E12"/>
   </mergeCells>
   <dataValidations count="18">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Unique" prompt="A value must be unique within the dataset" sqref="H19:H54" xr:uid="{00000000-0002-0000-0200-000000000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Unique" prompt="A value must be unique within the dataset" sqref="H18:H53" xr:uid="{00000000-0002-0000-0200-000000000000}">
       <formula1>"true,false"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C19:C54" xr:uid="{00000000-0002-0000-0200-000001000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C18:C53" xr:uid="{00000000-0002-0000-0200-000001000000}">
       <formula1>"string,number,integer,boolean,array,object,timestamp,date,time,map,vector"</formula1>
     </dataValidation>
-    <dataValidation allowBlank="1" sqref="B19:B54 J19:L54 O19:W54 Y19:AM54 AR19:AS54 AU19:AZ54" xr:uid="{00000000-0002-0000-0200-000002000000}"/>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Required" prompt="Is this a required field (true) or can it be optional (false)" sqref="G19:G54" xr:uid="{00000000-0002-0000-0200-000003000000}">
+    <dataValidation allowBlank="1" sqref="B18:B53 J18:L53 O18:W53 Y18:AM53 AR18:AS53 AU18:AZ53" xr:uid="{00000000-0002-0000-0200-000002000000}"/>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Required" prompt="Is this a required field (true) or can it be optional (false)" sqref="G18:G53" xr:uid="{00000000-0002-0000-0200-000003000000}">
       <formula1>"true,false"</formula1>
     </dataValidation>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Schema Name" prompt="The name of the schema (e.g., table) must match the Sheet name &quot;Schema &lt;schema_name&gt;&quot;" sqref="B5:E6" xr:uid="{00000000-0002-0000-0200-000004000000}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Property" prompt="Name of the property._x000a_If you have structured objects (child properties), use the dot notation, e.g., address.street._x000a_If you have array structures, use the [] notation, e.g., credit_cards[].number." sqref="A18" xr:uid="{00000000-0002-0000-0200-000005000000}"/>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Authoritative Definition Type" prompt="Type of definition for authority. Valid values are: businessDefinition, transformationImplementation, videoTutorial, tutorial, and implementation._x000a_ Maps to first authoritativeDefinitions.type_x000a_" sqref="N19:N54" xr:uid="{00000000-0002-0000-0200-000006000000}">
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Schema Name" prompt="The name of the schema (e.g., table) must match the Sheet name &quot;Schema &lt;schema_name&gt;&quot;" sqref="B5:E5" xr:uid="{00000000-0002-0000-0200-000004000000}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Property" prompt="Name of the property._x000a_If you have structured objects (child properties), use the dot notation, e.g., address.street._x000a_If you have array structures, use the [] notation, e.g., credit_cards[].number." sqref="A17" xr:uid="{00000000-0002-0000-0200-000005000000}"/>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Authoritative Definition Type" prompt="Type of definition for authority. Valid values are: businessDefinition, transformationImplementation, videoTutorial, tutorial, and implementation._x000a_ Maps to first authoritativeDefinitions.type_x000a_" sqref="N18:N53" xr:uid="{00000000-0002-0000-0200-000006000000}">
       <formula1>"businessDefinition,canonicalUrl,glossary,implementation,ontology,taxonomy,transformationImplementation,tutorial,videoTutorial"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="I19:I54" xr:uid="{00000000-0002-0000-0200-000007000000}">
+    <dataValidation type="list" allowBlank="1" sqref="I18:I53" xr:uid="{00000000-0002-0000-0200-000007000000}">
       <formula1>"confidential,restricted,public"</formula1>
     </dataValidation>
-    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Authoritative Definition URL" prompt="Links to sources that provide more details on the element; examples would be a link to privacy statement, terms and conditions, license agreements, data catalog, or another tool._x000a__x000a_Maps to first authoritativeDefinitions.url_x000a_" sqref="M19:M54" xr:uid="{00000000-0002-0000-0200-000008000000}"/>
-    <dataValidation type="list" allowBlank="1" sqref="X19:X54" xr:uid="{00000000-0002-0000-0200-000009000000}">
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Authoritative Definition URL" prompt="Links to sources that provide more details on the element; examples would be a link to privacy statement, terms and conditions, license agreements, data catalog, or another tool._x000a__x000a_Maps to first authoritativeDefinitions.url_x000a_" sqref="M18:M53" xr:uid="{00000000-0002-0000-0200-000008000000}"/>
+    <dataValidation type="list" allowBlank="1" sqref="X18:X53" xr:uid="{00000000-0002-0000-0200-000009000000}">
       <formula1>"TRUE,FALSE"</formula1>
     </dataValidation>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Comments" prompt="Use this for internal comments, open questions, discussion points. _x000a_This will not become part of the ODCS YAML." sqref="AW18" xr:uid="{00000000-0002-0000-0200-00000A000000}"/>
-    <dataValidation type="list" allowBlank="1" sqref="K19:K105" xr:uid="{00000000-0002-0000-0200-00000B000000}">
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Comments" prompt="Use this for internal comments, open questions, discussion points. _x000a_This will not become part of the ODCS YAML." sqref="AW17" xr:uid="{00000000-0002-0000-0200-00000A000000}"/>
+    <dataValidation type="list" allowBlank="1" sqref="K18:K104" xr:uid="{00000000-0002-0000-0200-00000B000000}">
       <formula1>"column,measure,dimension"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="L19:L105 AQ19:AQ102 AT19:AT102" xr:uid="{00000000-0002-0000-0200-00000C000000}">
+    <dataValidation type="list" allowBlank="1" sqref="L18:L104 AQ18:AQ101 AT18:AT101" xr:uid="{00000000-0002-0000-0200-00000C000000}">
       <formula1>"true,false"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B16:E16" xr:uid="{00000000-0002-0000-0200-00000D000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B15:E15" xr:uid="{00000000-0002-0000-0200-00000D000000}">
       <formula1>"true,false"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="AO19:AO102" xr:uid="{00000000-0002-0000-0200-00000E000000}">
+    <dataValidation type="list" allowBlank="1" sqref="AO18:AO101" xr:uid="{00000000-0002-0000-0200-00000E000000}">
       <formula1>"bfloat16,binary,float16,float32,float64,int8,uint8"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="AP19:AP102" xr:uid="{00000000-0002-0000-0200-00000F000000}">
+    <dataValidation type="list" allowBlank="1" sqref="AP18:AP101" xr:uid="{00000000-0002-0000-0200-00000F000000}">
       <formula1>"cosine,dotProduct,euclidean,hamming,manhattan"</formula1>
     </dataValidation>
-    <dataValidation type="whole" operator="greaterThanOrEqual" allowBlank="1" sqref="AN19:AN102" xr:uid="{00000000-0002-0000-0200-000010000000}">
+    <dataValidation type="whole" operator="greaterThanOrEqual" allowBlank="1" sqref="AN18:AN101" xr:uid="{00000000-0002-0000-0200-000010000000}">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B8:E8" xr:uid="{2DDE5C54-E084-1D42-BC0B-A6C800321056}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B7:E7" xr:uid="{3B9567C6-D3FB-7E46-9AF7-BBD3299CAA94}">
       <formula1>"object,blob"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>